<commit_message>
Regenerate the FINALE SAUCE BOM docs with clickable, resolving Mouser and datasheet links
</commit_message>
<xml_diff>
--- a/docs/FINALE_SAUCE_BOM.xlsx
+++ b/docs/FINALE_SAUCE_BOM.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -17,6 +17,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -34,9 +40,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -45,7 +52,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -57,12 +64,12 @@
     <col min="6" max="6" width="60" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="60" customWidth="1"/>
-    <col min="9" max="9" width="60" customWidth="1"/>
+    <col min="9" max="9" width="49" customWidth="1"/>
     <col min="10" max="10" width="60" customWidth="1"/>
     <col min="11" max="11" width="8" customWidth="1"/>
     <col min="12" max="12" width="29" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
-    <col min="14" max="14" width="8" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1"/>
     <col min="15" max="15" width="22" customWidth="1"/>
     <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="11" customWidth="1"/>
@@ -243,14 +250,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/560112116009.pdf</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/560112116009</t>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=560112116009</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -353,14 +360,14 @@
           <t xml:space="preserve">0402 (1005 metric)</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL05B104KO5NNN</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05B104KO5NNNC</t>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05B104KO5NNNC</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -459,14 +466,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-2102ELF</t>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-2102ELF</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -569,14 +576,14 @@
           <t xml:space="preserve">0402</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.vishay.com/docs/20035/dcrcwe3.pdf</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW04023R32FKED</t>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW04023R32FKED</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -679,14 +686,14 @@
           <t xml:space="preserve">Tray</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/85/1/qth.pdf</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samtec/QTH-060-01-L-D-A</t>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=QTH-060-01-L-D-A</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -785,14 +792,14 @@
           <t xml:space="preserve">VSSOP-8</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/sn74lvc1g74</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/SN74LVC1G74DCUR</t>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=SN74LVC1G74DCUR</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -891,14 +898,14 @@
           <t xml:space="preserve">SOT23-6</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/tps22917</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS22917LDBVR</t>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS22917LDBVR</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -997,14 +1004,14 @@
           <t xml:space="preserve">SOT-23-3</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.onsemi.com/pub/Collateral/NDS7002A-D.PDF</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/onsemi/2N7002</t>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=2N7002</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1103,14 +1110,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.te.com/commerce/DocumentDelivery/DDEController?Action=srchrtrv&amp;DocNm=1622877&amp;DocType=Customer+Drawing&amp;DocLang=English&amp;PartCntxt=1622877-2</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/TE-Connectivity-Holsworthy/CRG0603F1M0-10</t>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CRG0603F1M0-10</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1213,14 +1220,14 @@
           <t xml:space="preserve">1206 (3216 metric)</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL31A106KBHNNN</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL31A106KBHNNNE</t>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL31A106KBHNNNE</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1319,14 +1326,14 @@
           <t xml:space="preserve">VQFN-16</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/bq24075</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/BQ24074RGTT</t>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=BQ24074RGTT</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1425,14 +1432,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/560112116004.pdf</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/560112116004</t>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=560112116004</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1535,14 +1542,14 @@
           <t xml:space="preserve">0603 (1608 metric)</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL10A225KO8NNN</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL10A225KO8NNNC</t>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL10A225KO8NNNC</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1641,14 +1648,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://industrial.panasonic.com/cdbs/www-data/pdf/RDO0000/RDO0000C334.pdf</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Panasonic/ERJ-H3EF1022V</t>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=ERJ-H3EF1022V</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1751,14 +1758,14 @@
           <t xml:space="preserve">TSSOP-16</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/sn74lvc138a-ep</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/SN74LVC138AQPWREP</t>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=SN74LVC138AQPWREP</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1857,14 +1864,14 @@
           <t xml:space="preserve">Bulk</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/61300811121.pdf</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/61300811121</t>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=61300811121</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1963,14 +1970,14 @@
           <t xml:space="preserve">0402 (1005 metric)</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL05B102KB5NNN</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05B102KB5NNNC</t>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05B102KB5NNNC</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2069,14 +2076,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.vishay.com/docs/20035/dcrcwe3.pdf</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW0603249KFKEC</t>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW0603249KFKEC</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2179,14 +2186,14 @@
           <t xml:space="preserve">Reel</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/74438357010.pdf</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/74438357010</t>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=74438357010</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2289,14 +2296,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/317/1/ASC_MR.pdf</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Walsin/MR06X4703FTL</t>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=MR06X4703FTL</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2399,14 +2406,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://industrial.panasonic.com/cdbs/www-data/pdf/RDP0000/AOA0000C334.pdf</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Panasonic/ERJ-S03F1002V</t>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=ERJ-S03F1002V</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2509,14 +2516,14 @@
           <t xml:space="preserve">SOT-23-6</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/tps22918-q1</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS22918TDBVRQ1</t>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2615,14 +2622,14 @@
           <t xml:space="preserve">SOT-353-5</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/catalog/specsheets/diod-s-a0011233448-1.pdf</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Diodes-Incorporated/74AHC1G32QSE-7</t>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=74AHC1G32QSE-7</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2721,14 +2728,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://industrial.panasonic.com/cdbs/www-data/pdf/RDO0000/AOA0000C331.pdf</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Panasonic/ERJ-P03F1101V</t>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=ERJ-P03F1101V</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2831,14 +2838,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-4422ELF</t>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-4422ELF</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2941,14 +2948,14 @@
           <t xml:space="preserve">Reel</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/74439346068.pdf</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/74439346068</t>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=74439346068</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3051,14 +3058,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/317/1/ASC_MR.pdf</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Walsin/MR06X47R0FTL</t>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=MR06X47R0FTL</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -3161,14 +3168,14 @@
           <t xml:space="preserve">SOT-563-6</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/tps61023</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS61023DRLT</t>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS61023DRLT</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3267,14 +3274,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-3162ELF</t>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-3162ELF</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -3377,14 +3384,14 @@
           <t xml:space="preserve">3.2 mm x 2.5 mm</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/184/1/abm8.pdf</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/ABRACON/ABM8-25.000MHZ-B2-T</t>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=ABM8-25.000MHZ-B2-T</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3483,14 +3490,14 @@
           <t xml:space="preserve">Bulk</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/315/1/EG1218.pdf</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/E-Switch/EG1218</t>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=EG1218</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3585,12 +3592,12 @@
         </is>
       </c>
       <c r="G33"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/datasheet/3/167/1/Scotch_300_Series_Barricade_Tapes_Data_Sheet_78_8125_9670_4_F.pdf</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.adafruit.com/product/358</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.adafruit.com/product/358</t>
         </is>
@@ -3606,14 +3613,10 @@
           <t xml:space="preserve">Details</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">United States</t>
-        </is>
-      </c>
+      <c r="M33"/>
       <c r="N33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mouser</t>
+          <t xml:space="preserve">Adafruit</t>
         </is>
       </c>
       <c r="O33"/>
@@ -3641,9 +3644,7 @@
       <c r="W33">
         <v>59.85</v>
       </c>
-      <c r="X33">
-        <v>0</v>
-      </c>
+      <c r="X33"/>
       <c r="Y33">
         <v>0</v>
       </c>
@@ -3685,14 +3686,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://industrial.panasonic.com/cdbs/www-data/pdf/RDO0000/RDO0000C334.pdf</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Panasonic/ERJ-H3EF1872V</t>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=ERJ-H3EF1872V</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3795,14 +3796,14 @@
           <t xml:space="preserve">0402</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.vishay.com/docs/20035/dcrcwe3.pdf</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW04024K12FKED</t>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW04024K12FKED</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3905,14 +3906,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-4642ELF</t>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-4642ELF</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -4015,14 +4016,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-1181ELF</t>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-1181ELF</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -4125,14 +4126,14 @@
           <t xml:space="preserve">SOT-23-6</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/tps3700</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS3700DDCR</t>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS3700DDCR</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -4231,14 +4232,14 @@
           <t xml:space="preserve">0805 (2012 metric)</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL21A106KOQNNN</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL21A106KOQNNNE</t>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL21A106KOQNNNE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4337,14 +4338,14 @@
           <t xml:space="preserve">SOT-23-5</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/ts5a3166</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TS5A3166DBVR</t>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=TS5A3166DBVR</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -4443,14 +4444,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/560112116040.pdf</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/560112116040</t>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=560112116040</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4553,14 +4554,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-4700ELF</t>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-4700ELF</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -4663,14 +4664,14 @@
           <t xml:space="preserve">Bulk</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/61300411121.pdf</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/61300411121</t>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=61300411121</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4769,14 +4770,14 @@
           <t xml:space="preserve">SOT-23-6</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.analog.com/MAX4995B/datasheet</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Analog-Devices-Maxim-Integrated/MAX4995BAUT%2bT</t>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=MAX4995BAUT_T</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4875,14 +4876,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.vishay.com/docs/20008/dcrcw.pdf</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW0603133KFKTA</t>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW0603133KFKTA</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4985,14 +4986,14 @@
           <t xml:space="preserve">SOT-23-5</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/sn74lvc1g08</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/SN74LVC1G08DBVT</t>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=SN74LVC1G08DBVT</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -5091,14 +5092,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-22R0ELF</t>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-22R0ELF</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -5201,14 +5202,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-3300ELF</t>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-3300ELF</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5311,14 +5312,14 @@
           <t xml:space="preserve">0402 (1005 metric)</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL05B222KB5NNN</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05B222KB5NNNC</t>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05B222KB5NNNC</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -5417,14 +5418,14 @@
           <t xml:space="preserve">VQFN-HR-10</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/tps25947</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS259470LRPWR</t>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS259470LRPWR</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5523,14 +5524,14 @@
           <t xml:space="preserve">SOT-583-8</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/tps62933p</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS62933PDRLR</t>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS62933PDRLR</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -5629,14 +5630,14 @@
           <t xml:space="preserve">0402</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/catalog/specsheets/YAGEO_PYu_RC_Group_51_RoHS_L_12.pdf</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/YAGEO/RC0402FR-0710KL</t>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=RC0402FR-0710KL</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -5735,14 +5736,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-5101ELF</t>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-5101ELF</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -5845,14 +5846,14 @@
           <t xml:space="preserve">0603 (1608 metric)</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/150060RS75000.pdf</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/150060RS75000</t>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=150060RS75000</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -5951,14 +5952,14 @@
           <t xml:space="preserve">SOD-923-2</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.onsemi.com/pub/Collateral/ESD9X3.3ST5G-D.PDF</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/onsemi/ESD9X5.0ST5G</t>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=ESD9X5.0ST5G</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -6057,14 +6058,14 @@
           <t xml:space="preserve">LQFP-144</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.st.com/resource/en/datasheet/stm32h753vi.pdf</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/STMicroelectronics/STM32H753ZIT6</t>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=STM32H753ZIT6</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -6163,14 +6164,14 @@
           <t xml:space="preserve">Tray</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/201/1/1043.pdf</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Keystone-Electronics/1043</t>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=1043</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -6269,14 +6270,14 @@
           <t xml:space="preserve">Reel</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://ckswitches.com/media/1471/pts645.pdf</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/CK/PTS645SM43SMTR92-LFS</t>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=PTS645SM43SMTR92LFS</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -6371,14 +6372,14 @@
           <t xml:space="preserve">Reel</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/srp7028a.pdf</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/SRP7028A-4R7M</t>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=SRP7028A-4R7M</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -6477,14 +6478,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/72/1/PYU_RT_1_TO_0_01_ROHS_L.pdf</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/YAGEO/RT0603BRD0794K2L</t>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=RT0603BRD0794K2L</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -6587,14 +6588,14 @@
           <t xml:space="preserve">0402 (1005 metric)</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL05C220JB5NNN</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05C220JB5NNNC</t>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05C220JB5NNNC</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -6693,14 +6694,14 @@
           <t xml:space="preserve">0402 (1005 metric)</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL05C100JB5NNN</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05C100JB5NNNC</t>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05C100JB5NNNC</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -6799,14 +6800,14 @@
           <t xml:space="preserve">0402 (1005 metric)</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL05C750JB5NNN</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05C750JB5NNNC</t>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05C750JB5NNNC</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -6901,14 +6902,14 @@
           <t xml:space="preserve">0805 (2012 metric)</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://s3.us-west-2.amazonaws.com/catsy.557/Dialight_datasheet_599_Single-Color_0805_2_Taiwan.pdf</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Dialight/599-0160-137F</t>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=599-0160-137F</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -7007,14 +7008,14 @@
           <t xml:space="preserve">1206 (3216 metric)</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL31A226KAHNNN</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL31A226KAHNNNE</t>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL31A226KAHNNNE</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -7113,14 +7114,14 @@
           <t xml:space="preserve">VQFN-12</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/tps2121</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS2121RUXR</t>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS2121RUXR</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -7219,14 +7220,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-6652ELF</t>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-6652ELF</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -7329,14 +7330,14 @@
           <t xml:space="preserve">Top-Mount</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/catalog/specsheets/Global_Connector_Technology_usb4105.pdf</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/GCT/USB4105-GF-A</t>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=USB4105-GF-A</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -7435,14 +7436,14 @@
           <t xml:space="preserve">0805 (2012 metric)</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL21A475KAQNNN</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL21A475KAQNNNE</t>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL21A475KAQNNNE</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -7541,14 +7542,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/catalog/specsheets/YAGEO_PYu_RC_Group_51_RoHS_L_12.pdf</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/YAGEO/RC0603FR-07220RL</t>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=RC0603FR-07220RL</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -7647,14 +7648,14 @@
           <t xml:space="preserve">SC-59-3 (SOT-23-3)</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/tpd2e009</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPD2E009DBZR</t>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=TPD2E009DBZR</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -7753,14 +7754,14 @@
           <t xml:space="preserve">0603 (1608 metric)</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/150060GS75000.pdf</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/150060GS75000</t>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=150060GS75000</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -7859,14 +7860,14 @@
           <t xml:space="preserve">0402 (1005 metric)</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL05B332KB5NNN</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05B332KB5NNNC</t>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05B332KB5NNNC</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -7965,14 +7966,14 @@
           <t xml:space="preserve">SOT-5X3-5</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="H74" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/sn74ahc1g125</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/SN74AHC1G125DRLR</t>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=SN74AHC1G125DRLR</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -8067,14 +8068,14 @@
         </is>
       </c>
       <c r="G75"/>
-      <c r="H75" t="inlineStr">
+      <c r="H75" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/catalog/specsheets/Yamaichi%20Electronics_08162018_IC51-0644-807_H.pdf</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Yamaichi-Electronics/IC51-0644-807</t>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=IC51-0644-807</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -8173,14 +8174,14 @@
           <t xml:space="preserve">SOT-5X3-5</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
+      <c r="H76" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/sn74lvc1gu04</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/SN74LVC1GU04DRLR</t>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=SN74LVC1GU04DRLR</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -8279,14 +8280,14 @@
           <t xml:space="preserve">0603 (1608 metric)</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
+      <c r="H77" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL10A475KO8NNN</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL10A475KO8NNNC</t>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL10A475KO8NNNC</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -8385,14 +8386,14 @@
           <t xml:space="preserve">VSSOP-8</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr">
+      <c r="H78" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.ti.com/lit/gpn/txs0102</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TXS0102DCUR</t>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=TXS0102DCUR</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -8491,14 +8492,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr">
+      <c r="H79" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/508/1/PYu-AC_51_RoHS_L_11.pdf</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/YAGEO/AC0603FR-07255KL</t>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=AC0603FR-07255KL</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -8601,14 +8602,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
+      <c r="H80" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.vishay.com/docs/20035/dcrcwe3.pdf</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW06035K05FKEA</t>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW06035K05FKEA</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -8711,14 +8712,14 @@
           <t xml:space="preserve">Reel</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
+      <c r="H81" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://ckswitches.com/media/1422/js.pdf</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/CK/JS102011SAQN</t>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=JS102011SAQN</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -8817,14 +8818,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
+      <c r="H82" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.rohm.com/datasheet?p=KTR03EZPF</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/ROHM-Semiconductor/KTR03EZPF3403</t>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=KTR03EZPF3403</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -8927,14 +8928,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
+      <c r="H83" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.vishay.com/docs/20008/dcrcw.pdf</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW06033R32FKTA</t>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW06033R32FKTA</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -9037,14 +9038,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="H84" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/40/1/cr.pdf</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-6800ELF</t>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-6800ELF</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -9147,14 +9148,14 @@
           <t xml:space="preserve">0805 (2012 metric)</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="H85" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/742792022.pdf</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/742792022</t>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=742792022</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -9253,14 +9254,14 @@
           <t xml:space="preserve">0603</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H86" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.we-online.com/components/products/datasheet/560112116151.pdf</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/560112116151</t>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=560112116151</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -9363,14 +9364,14 @@
           <t xml:space="preserve">0402</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
+      <c r="H87" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://industrial.panasonic.com/cdbs/www-data/pdf/RDO0000/AOA0000C331.pdf</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Panasonic/ERJ-PA2F1242X</t>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=ERJ-PA2F1242X</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -9473,14 +9474,14 @@
           <t xml:space="preserve">Tray</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr">
+      <c r="H88" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.mouser.com/datasheet/3/85/1/qsh.pdf</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samtec/QSH-060-01-H-D-A</t>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=QSH-060-01-H-D-A</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -9579,14 +9580,14 @@
           <t xml:space="preserve">0603 (1608 metric)</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr">
+      <c r="H89" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://weblib.samsungsem.com/mlcc/mlcc-ec-data-sheet.do?partNumber=CL10A105KB8NNN</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL10A105KB8NNNC</t>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.mouser.com/c/?q=CL10A105KB8NNNC</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -9653,5 +9654,183 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:Z89"/>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1"/>
+    <hyperlink ref="I2" r:id="rId2"/>
+    <hyperlink ref="H3" r:id="rId3"/>
+    <hyperlink ref="I3" r:id="rId4"/>
+    <hyperlink ref="H4" r:id="rId5"/>
+    <hyperlink ref="I4" r:id="rId6"/>
+    <hyperlink ref="H5" r:id="rId7"/>
+    <hyperlink ref="I5" r:id="rId8"/>
+    <hyperlink ref="H6" r:id="rId9"/>
+    <hyperlink ref="I6" r:id="rId10"/>
+    <hyperlink ref="H7" r:id="rId11"/>
+    <hyperlink ref="I7" r:id="rId12"/>
+    <hyperlink ref="H8" r:id="rId13"/>
+    <hyperlink ref="I8" r:id="rId14"/>
+    <hyperlink ref="H9" r:id="rId15"/>
+    <hyperlink ref="I9" r:id="rId16"/>
+    <hyperlink ref="H10" r:id="rId17"/>
+    <hyperlink ref="I10" r:id="rId18"/>
+    <hyperlink ref="H11" r:id="rId19"/>
+    <hyperlink ref="I11" r:id="rId20"/>
+    <hyperlink ref="H12" r:id="rId21"/>
+    <hyperlink ref="I12" r:id="rId22"/>
+    <hyperlink ref="H13" r:id="rId23"/>
+    <hyperlink ref="I13" r:id="rId24"/>
+    <hyperlink ref="H14" r:id="rId25"/>
+    <hyperlink ref="I14" r:id="rId26"/>
+    <hyperlink ref="H15" r:id="rId27"/>
+    <hyperlink ref="I15" r:id="rId28"/>
+    <hyperlink ref="H16" r:id="rId29"/>
+    <hyperlink ref="I16" r:id="rId30"/>
+    <hyperlink ref="H17" r:id="rId31"/>
+    <hyperlink ref="I17" r:id="rId32"/>
+    <hyperlink ref="H18" r:id="rId33"/>
+    <hyperlink ref="I18" r:id="rId34"/>
+    <hyperlink ref="H19" r:id="rId35"/>
+    <hyperlink ref="I19" r:id="rId36"/>
+    <hyperlink ref="H20" r:id="rId37"/>
+    <hyperlink ref="I20" r:id="rId38"/>
+    <hyperlink ref="H21" r:id="rId39"/>
+    <hyperlink ref="I21" r:id="rId40"/>
+    <hyperlink ref="H22" r:id="rId41"/>
+    <hyperlink ref="I22" r:id="rId42"/>
+    <hyperlink ref="H23" r:id="rId43"/>
+    <hyperlink ref="I23" r:id="rId44"/>
+    <hyperlink ref="H24" r:id="rId45"/>
+    <hyperlink ref="I24" r:id="rId46"/>
+    <hyperlink ref="H25" r:id="rId47"/>
+    <hyperlink ref="I25" r:id="rId48"/>
+    <hyperlink ref="H26" r:id="rId49"/>
+    <hyperlink ref="I26" r:id="rId50"/>
+    <hyperlink ref="H27" r:id="rId51"/>
+    <hyperlink ref="I27" r:id="rId52"/>
+    <hyperlink ref="H28" r:id="rId53"/>
+    <hyperlink ref="I28" r:id="rId54"/>
+    <hyperlink ref="H29" r:id="rId55"/>
+    <hyperlink ref="I29" r:id="rId56"/>
+    <hyperlink ref="H30" r:id="rId57"/>
+    <hyperlink ref="I30" r:id="rId58"/>
+    <hyperlink ref="H31" r:id="rId59"/>
+    <hyperlink ref="I31" r:id="rId60"/>
+    <hyperlink ref="H32" r:id="rId61"/>
+    <hyperlink ref="I32" r:id="rId62"/>
+    <hyperlink ref="H33" r:id="rId63"/>
+    <hyperlink ref="I33" r:id="rId64"/>
+    <hyperlink ref="H34" r:id="rId65"/>
+    <hyperlink ref="I34" r:id="rId66"/>
+    <hyperlink ref="H35" r:id="rId67"/>
+    <hyperlink ref="I35" r:id="rId68"/>
+    <hyperlink ref="H36" r:id="rId69"/>
+    <hyperlink ref="I36" r:id="rId70"/>
+    <hyperlink ref="H37" r:id="rId71"/>
+    <hyperlink ref="I37" r:id="rId72"/>
+    <hyperlink ref="H38" r:id="rId73"/>
+    <hyperlink ref="I38" r:id="rId74"/>
+    <hyperlink ref="H39" r:id="rId75"/>
+    <hyperlink ref="I39" r:id="rId76"/>
+    <hyperlink ref="H40" r:id="rId77"/>
+    <hyperlink ref="I40" r:id="rId78"/>
+    <hyperlink ref="H41" r:id="rId79"/>
+    <hyperlink ref="I41" r:id="rId80"/>
+    <hyperlink ref="H42" r:id="rId81"/>
+    <hyperlink ref="I42" r:id="rId82"/>
+    <hyperlink ref="H43" r:id="rId83"/>
+    <hyperlink ref="I43" r:id="rId84"/>
+    <hyperlink ref="H44" r:id="rId85"/>
+    <hyperlink ref="I44" r:id="rId86"/>
+    <hyperlink ref="H45" r:id="rId87"/>
+    <hyperlink ref="I45" r:id="rId88"/>
+    <hyperlink ref="H46" r:id="rId89"/>
+    <hyperlink ref="I46" r:id="rId90"/>
+    <hyperlink ref="H47" r:id="rId91"/>
+    <hyperlink ref="I47" r:id="rId92"/>
+    <hyperlink ref="H48" r:id="rId93"/>
+    <hyperlink ref="I48" r:id="rId94"/>
+    <hyperlink ref="H49" r:id="rId95"/>
+    <hyperlink ref="I49" r:id="rId96"/>
+    <hyperlink ref="H50" r:id="rId97"/>
+    <hyperlink ref="I50" r:id="rId98"/>
+    <hyperlink ref="H51" r:id="rId99"/>
+    <hyperlink ref="I51" r:id="rId100"/>
+    <hyperlink ref="H52" r:id="rId101"/>
+    <hyperlink ref="I52" r:id="rId102"/>
+    <hyperlink ref="H53" r:id="rId103"/>
+    <hyperlink ref="I53" r:id="rId104"/>
+    <hyperlink ref="H54" r:id="rId105"/>
+    <hyperlink ref="I54" r:id="rId106"/>
+    <hyperlink ref="H55" r:id="rId107"/>
+    <hyperlink ref="I55" r:id="rId108"/>
+    <hyperlink ref="H56" r:id="rId109"/>
+    <hyperlink ref="I56" r:id="rId110"/>
+    <hyperlink ref="H57" r:id="rId111"/>
+    <hyperlink ref="I57" r:id="rId112"/>
+    <hyperlink ref="H58" r:id="rId113"/>
+    <hyperlink ref="I58" r:id="rId114"/>
+    <hyperlink ref="H59" r:id="rId115"/>
+    <hyperlink ref="I59" r:id="rId116"/>
+    <hyperlink ref="H60" r:id="rId117"/>
+    <hyperlink ref="I60" r:id="rId118"/>
+    <hyperlink ref="H61" r:id="rId119"/>
+    <hyperlink ref="I61" r:id="rId120"/>
+    <hyperlink ref="H62" r:id="rId121"/>
+    <hyperlink ref="I62" r:id="rId122"/>
+    <hyperlink ref="H63" r:id="rId123"/>
+    <hyperlink ref="I63" r:id="rId124"/>
+    <hyperlink ref="H64" r:id="rId125"/>
+    <hyperlink ref="I64" r:id="rId126"/>
+    <hyperlink ref="H65" r:id="rId127"/>
+    <hyperlink ref="I65" r:id="rId128"/>
+    <hyperlink ref="H66" r:id="rId129"/>
+    <hyperlink ref="I66" r:id="rId130"/>
+    <hyperlink ref="H67" r:id="rId131"/>
+    <hyperlink ref="I67" r:id="rId132"/>
+    <hyperlink ref="H68" r:id="rId133"/>
+    <hyperlink ref="I68" r:id="rId134"/>
+    <hyperlink ref="H69" r:id="rId135"/>
+    <hyperlink ref="I69" r:id="rId136"/>
+    <hyperlink ref="H70" r:id="rId137"/>
+    <hyperlink ref="I70" r:id="rId138"/>
+    <hyperlink ref="H71" r:id="rId139"/>
+    <hyperlink ref="I71" r:id="rId140"/>
+    <hyperlink ref="H72" r:id="rId141"/>
+    <hyperlink ref="I72" r:id="rId142"/>
+    <hyperlink ref="H73" r:id="rId143"/>
+    <hyperlink ref="I73" r:id="rId144"/>
+    <hyperlink ref="H74" r:id="rId145"/>
+    <hyperlink ref="I74" r:id="rId146"/>
+    <hyperlink ref="H75" r:id="rId147"/>
+    <hyperlink ref="I75" r:id="rId148"/>
+    <hyperlink ref="H76" r:id="rId149"/>
+    <hyperlink ref="I76" r:id="rId150"/>
+    <hyperlink ref="H77" r:id="rId151"/>
+    <hyperlink ref="I77" r:id="rId152"/>
+    <hyperlink ref="H78" r:id="rId153"/>
+    <hyperlink ref="I78" r:id="rId154"/>
+    <hyperlink ref="H79" r:id="rId155"/>
+    <hyperlink ref="I79" r:id="rId156"/>
+    <hyperlink ref="H80" r:id="rId157"/>
+    <hyperlink ref="I80" r:id="rId158"/>
+    <hyperlink ref="H81" r:id="rId159"/>
+    <hyperlink ref="I81" r:id="rId160"/>
+    <hyperlink ref="H82" r:id="rId161"/>
+    <hyperlink ref="I82" r:id="rId162"/>
+    <hyperlink ref="H83" r:id="rId163"/>
+    <hyperlink ref="I83" r:id="rId164"/>
+    <hyperlink ref="H84" r:id="rId165"/>
+    <hyperlink ref="I84" r:id="rId166"/>
+    <hyperlink ref="H85" r:id="rId167"/>
+    <hyperlink ref="I85" r:id="rId168"/>
+    <hyperlink ref="H86" r:id="rId169"/>
+    <hyperlink ref="I86" r:id="rId170"/>
+    <hyperlink ref="H87" r:id="rId171"/>
+    <hyperlink ref="I87" r:id="rId172"/>
+    <hyperlink ref="H88" r:id="rId173"/>
+    <hyperlink ref="I88" r:id="rId174"/>
+    <hyperlink ref="H89" r:id="rId175"/>
+    <hyperlink ref="I89" r:id="rId176"/>
+  </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restore the original supplied purchase links (revert the wrongly-generated /c/?q= rewrite); keep them as clickable hyperlinks
</commit_message>
<xml_diff>
--- a/docs/FINALE_SAUCE_BOM.xlsx
+++ b/docs/FINALE_SAUCE_BOM.xlsx
@@ -64,13 +64,13 @@
     <col min="6" max="6" width="60" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="60" customWidth="1"/>
-    <col min="9" max="9" width="49" customWidth="1"/>
+    <col min="9" max="9" width="60" customWidth="1"/>
     <col min="10" max="10" width="60" customWidth="1"/>
     <col min="11" max="11" width="8" customWidth="1"/>
     <col min="12" max="12" width="29" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
     <col min="14" max="14" width="10" customWidth="1"/>
-    <col min="15" max="15" width="22" customWidth="1"/>
+    <col min="15" max="15" width="10" customWidth="1"/>
     <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="11" customWidth="1"/>
     <col min="18" max="18" width="9" customWidth="1"/>
@@ -257,7 +257,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=560112116009</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/560112116009</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -285,11 +285,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-560112116009</t>
-        </is>
-      </c>
+      <c r="O2"/>
       <c r="P2">
         <v>0.11</v>
       </c>
@@ -367,7 +363,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05B104KO5NNNC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05B104KO5NNNC</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -391,11 +387,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL05B104KO5NNNC</t>
-        </is>
-      </c>
+      <c r="O3"/>
       <c r="P3">
         <v>0.1</v>
       </c>
@@ -473,7 +465,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-2102ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-2102ELF</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -501,11 +493,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603FX-2102ELF</t>
-        </is>
-      </c>
+      <c r="O4"/>
       <c r="P4">
         <v>0.1</v>
       </c>
@@ -583,7 +571,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW04023R32FKED</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW04023R32FKED</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -611,11 +599,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">71-CRCW0402-3.32-E3</t>
-        </is>
-      </c>
+      <c r="O5"/>
       <c r="P5">
         <v>0.1</v>
       </c>
@@ -693,7 +677,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=QTH-060-01-L-D-A</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samtec/QTH-060-01-L-D-A</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -717,11 +701,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">200-QTH06001LDA</t>
-        </is>
-      </c>
+      <c r="O6"/>
       <c r="P6">
         <v>5.75</v>
       </c>
@@ -799,7 +779,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=SN74LVC1G74DCUR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/SN74LVC1G74DCUR</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -823,11 +803,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-SN74LVC1G74DCUR</t>
-        </is>
-      </c>
+      <c r="O7"/>
       <c r="P7">
         <v>0.6</v>
       </c>
@@ -905,7 +881,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS22917LDBVR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS22917LDBVR</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -929,11 +905,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-TPS22917LDBVR</t>
-        </is>
-      </c>
+      <c r="O8"/>
       <c r="P8">
         <v>0.52</v>
       </c>
@@ -1011,7 +983,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=2N7002</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/onsemi/2N7002</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1035,11 +1007,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">512-2N7002</t>
-        </is>
-      </c>
+      <c r="O9"/>
       <c r="P9">
         <v>1.09</v>
       </c>
@@ -1117,7 +1085,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CRG0603F1M0-10</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/TE-Connectivity-Holsworthy/CRG0603F1M0-10</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1145,11 +1113,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">279-CRG0603F1M0/10</t>
-        </is>
-      </c>
+      <c r="O10"/>
       <c r="P10">
         <v>0.24</v>
       </c>
@@ -1227,7 +1191,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL31A106KBHNNNE</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL31A106KBHNNNE</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1251,11 +1215,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL31A106KBHNNNE</t>
-        </is>
-      </c>
+      <c r="O11"/>
       <c r="P11">
         <v>0.36</v>
       </c>
@@ -1333,7 +1293,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=BQ24074RGTT</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/BQ24074RGTT</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1357,11 +1317,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-BQ24074RGTT</t>
-        </is>
-      </c>
+      <c r="O12"/>
       <c r="P12">
         <v>3.19</v>
       </c>
@@ -1439,7 +1395,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=560112116004</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/560112116004</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1467,11 +1423,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-560112116004</t>
-        </is>
-      </c>
+      <c r="O13"/>
       <c r="P13">
         <v>0.11</v>
       </c>
@@ -1549,7 +1501,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL10A225KO8NNNC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL10A225KO8NNNC</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1573,11 +1525,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL10A225KO8NNNC</t>
-        </is>
-      </c>
+      <c r="O14"/>
       <c r="P14">
         <v>0.1</v>
       </c>
@@ -1655,7 +1603,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=ERJ-H3EF1022V</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Panasonic/ERJ-H3EF1022V</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1683,11 +1631,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">667-ERJ-H3EF1022V</t>
-        </is>
-      </c>
+      <c r="O15"/>
       <c r="P15">
         <v>0.28</v>
       </c>
@@ -1765,7 +1709,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=SN74LVC138AQPWREP</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/SN74LVC138AQPWREP</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1789,11 +1733,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-N74LVC138AQPWREP</t>
-        </is>
-      </c>
+      <c r="O16"/>
       <c r="P16">
         <v>2.73</v>
       </c>
@@ -1871,7 +1811,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=61300811121</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/61300811121</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1895,11 +1835,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-61300811121</t>
-        </is>
-      </c>
+      <c r="O17"/>
       <c r="P17">
         <v>0.39</v>
       </c>
@@ -1977,7 +1913,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05B102KB5NNNC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05B102KB5NNNC</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2001,11 +1937,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL05B102KB5NNNC</t>
-        </is>
-      </c>
+      <c r="O18"/>
       <c r="P18">
         <v>0.1</v>
       </c>
@@ -2083,7 +2015,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW0603249KFKEC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW0603249KFKEC</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2111,11 +2043,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">71-CRCW0603249KFKEC</t>
-        </is>
-      </c>
+      <c r="O19"/>
       <c r="P19">
         <v>0.25</v>
       </c>
@@ -2193,7 +2121,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=74438357010</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/74438357010</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2221,11 +2149,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-74438357010</t>
-        </is>
-      </c>
+      <c r="O20"/>
       <c r="P20">
         <v>1.68</v>
       </c>
@@ -2303,7 +2227,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=MR06X4703FTL</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Walsin/MR06X4703FTL</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2331,11 +2255,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">791-MR06X4703FTL</t>
-        </is>
-      </c>
+      <c r="O21"/>
       <c r="P21">
         <v>0.13</v>
       </c>
@@ -2413,7 +2333,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=ERJ-S03F1002V</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Panasonic/ERJ-S03F1002V</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2441,11 +2361,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">667-ERJ-S03F1002V</t>
-        </is>
-      </c>
+      <c r="O22"/>
       <c r="P22">
         <v>0.23</v>
       </c>
@@ -2523,7 +2439,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS22918TDBVRQ1</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2547,11 +2463,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-TPS22918TDBVRQ1</t>
-        </is>
-      </c>
+      <c r="O23"/>
       <c r="P23">
         <v>0.76</v>
       </c>
@@ -2629,7 +2541,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=74AHC1G32QSE-7</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Diodes-Incorporated/74AHC1G32QSE-7</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2653,11 +2565,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">621-74AHC1G32QSE-7</t>
-        </is>
-      </c>
+      <c r="O24"/>
       <c r="P24">
         <v>0.14</v>
       </c>
@@ -2735,7 +2643,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=ERJ-P03F1101V</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Panasonic/ERJ-P03F1101V</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2763,11 +2671,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">667-ERJ-P03F1101V</t>
-        </is>
-      </c>
+      <c r="O25"/>
       <c r="P25">
         <v>0.31</v>
       </c>
@@ -2845,7 +2749,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-4422ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-4422ELF</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2873,11 +2777,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603FX-4422ELF</t>
-        </is>
-      </c>
+      <c r="O26"/>
       <c r="P26">
         <v>0.1</v>
       </c>
@@ -2955,7 +2855,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=74439346068</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/74439346068</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2983,11 +2883,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-74439346068</t>
-        </is>
-      </c>
+      <c r="O27"/>
       <c r="P27">
         <v>4.05</v>
       </c>
@@ -3065,7 +2961,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=MR06X47R0FTL</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Walsin/MR06X47R0FTL</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -3093,11 +2989,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">791-MR06X47R0FTL</t>
-        </is>
-      </c>
+      <c r="O28"/>
       <c r="P28">
         <v>0.13</v>
       </c>
@@ -3175,7 +3067,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS61023DRLT</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS61023DRLT</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3199,11 +3091,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-TPS61023DRLT</t>
-        </is>
-      </c>
+      <c r="O29"/>
       <c r="P29">
         <v>1.43</v>
       </c>
@@ -3281,7 +3169,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-3162ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-3162ELF</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -3309,11 +3197,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603FX-3162ELF</t>
-        </is>
-      </c>
+      <c r="O30"/>
       <c r="P30">
         <v>0.1</v>
       </c>
@@ -3391,7 +3275,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=ABM8-25.000MHZ-B2-T</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/ABRACON/ABM8-25.000MHZ-B2-T</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3415,11 +3299,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">815-ABM8-25-B2-T</t>
-        </is>
-      </c>
+      <c r="O31"/>
       <c r="P31">
         <v>0.5</v>
       </c>
@@ -3497,7 +3377,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=EG1218</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/E-Switch/EG1218</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3521,11 +3401,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">612-EG1218</t>
-        </is>
-      </c>
+      <c r="O32"/>
       <c r="P32">
         <v>0.71</v>
       </c>
@@ -3693,7 +3569,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=ERJ-H3EF1872V</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Panasonic/ERJ-H3EF1872V</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3721,11 +3597,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">667-ERJ-H3EF1872V</t>
-        </is>
-      </c>
+      <c r="O34"/>
       <c r="P34">
         <v>0.28</v>
       </c>
@@ -3803,7 +3675,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW04024K12FKED</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW04024K12FKED</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3831,11 +3703,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">71-CRCW0402-4.12K-E3</t>
-        </is>
-      </c>
+      <c r="O35"/>
       <c r="P35">
         <v>0.15</v>
       </c>
@@ -3913,7 +3781,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-4642ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-4642ELF</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3941,11 +3809,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603FX-4642ELF</t>
-        </is>
-      </c>
+      <c r="O36"/>
       <c r="P36">
         <v>0.1</v>
       </c>
@@ -4023,7 +3887,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-1181ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-1181ELF</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -4051,11 +3915,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603FX-1181ELF</t>
-        </is>
-      </c>
+      <c r="O37"/>
       <c r="P37">
         <v>0.1</v>
       </c>
@@ -4133,7 +3993,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS3700DDCR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS3700DDCR</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -4157,11 +4017,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-TPS3700DDCR</t>
-        </is>
-      </c>
+      <c r="O38"/>
       <c r="P38">
         <v>2.52</v>
       </c>
@@ -4239,7 +4095,7 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL21A106KOQNNNE</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL21A106KOQNNNE</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4263,11 +4119,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL21A106KOQNNNE</t>
-        </is>
-      </c>
+      <c r="O39"/>
       <c r="P39">
         <v>0.11</v>
       </c>
@@ -4345,7 +4197,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=TS5A3166DBVR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TS5A3166DBVR</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -4369,11 +4221,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-TS5A3166DBVR</t>
-        </is>
-      </c>
+      <c r="O40"/>
       <c r="P40">
         <v>0.43</v>
       </c>
@@ -4451,7 +4299,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=560112116040</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/560112116040</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4479,11 +4327,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-560112116040</t>
-        </is>
-      </c>
+      <c r="O41"/>
       <c r="P41">
         <v>0.11</v>
       </c>
@@ -4561,7 +4405,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-4700ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-4700ELF</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -4589,11 +4433,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603FX-4700ELF</t>
-        </is>
-      </c>
+      <c r="O42"/>
       <c r="P42">
         <v>0.1</v>
       </c>
@@ -4671,7 +4511,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=61300411121</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/61300411121</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4695,11 +4535,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-61300411121</t>
-        </is>
-      </c>
+      <c r="O43"/>
       <c r="P43">
         <v>0.19</v>
       </c>
@@ -4777,7 +4613,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=MAX4995BAUT_T</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Analog-Devices-Maxim-Integrated/MAX4995BAUT%2bT</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4801,11 +4637,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">700-MAX4995BAUTT</t>
-        </is>
-      </c>
+      <c r="O44"/>
       <c r="P44">
         <v>6.99</v>
       </c>
@@ -4883,7 +4715,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW0603133KFKTA</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW0603133KFKTA</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4911,11 +4743,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">71-CRCW0603-133K</t>
-        </is>
-      </c>
+      <c r="O45"/>
       <c r="P45">
         <v>0.16</v>
       </c>
@@ -4993,7 +4821,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=SN74LVC1G08DBVT</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/SN74LVC1G08DBVT</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -5017,11 +4845,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-SN74LVC1G08DBVT</t>
-        </is>
-      </c>
+      <c r="O46"/>
       <c r="P46">
         <v>0.9</v>
       </c>
@@ -5099,7 +4923,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-22R0ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-22R0ELF</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -5127,11 +4951,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603FX-22R0ELF</t>
-        </is>
-      </c>
+      <c r="O47"/>
       <c r="P47">
         <v>0.1</v>
       </c>
@@ -5209,7 +5029,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-3300ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-3300ELF</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5237,11 +5057,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603FX-3300ELF</t>
-        </is>
-      </c>
+      <c r="O48"/>
       <c r="P48">
         <v>0.1</v>
       </c>
@@ -5319,7 +5135,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05B222KB5NNNC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05B222KB5NNNC</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -5343,11 +5159,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL05B222KB5NNNC</t>
-        </is>
-      </c>
+      <c r="O49"/>
       <c r="P49">
         <v>0.1</v>
       </c>
@@ -5425,7 +5237,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS259470LRPWR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS259470LRPWR</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5449,11 +5261,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-TPS259470LRPWR</t>
-        </is>
-      </c>
+      <c r="O50"/>
       <c r="P50">
         <v>1.71</v>
       </c>
@@ -5531,7 +5339,7 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS62933PDRLR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS62933PDRLR</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -5555,11 +5363,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-TPS62933PDRLR</t>
-        </is>
-      </c>
+      <c r="O51"/>
       <c r="P51">
         <v>1.38</v>
       </c>
@@ -5637,7 +5441,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=RC0402FR-0710KL</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/YAGEO/RC0402FR-0710KL</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -5661,11 +5465,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">603-RC0402FR-0710KL</t>
-        </is>
-      </c>
+      <c r="O52"/>
       <c r="P52">
         <v>0.1</v>
       </c>
@@ -5743,7 +5543,7 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-5101ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-5101ELF</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -5771,11 +5571,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603FX-5101ELF</t>
-        </is>
-      </c>
+      <c r="O53"/>
       <c r="P53">
         <v>0.1</v>
       </c>
@@ -5853,7 +5649,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=150060RS75000</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/150060RS75000</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -5877,11 +5673,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-150060RS75000</t>
-        </is>
-      </c>
+      <c r="O54"/>
       <c r="P54">
         <v>0.16</v>
       </c>
@@ -5959,7 +5751,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=ESD9X5.0ST5G</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/onsemi/ESD9X5.0ST5G</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -5983,11 +5775,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">863-ESD9X5.0ST5G</t>
-        </is>
-      </c>
+      <c r="O55"/>
       <c r="P55">
         <v>0.16</v>
       </c>
@@ -6065,7 +5853,7 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=STM32H753ZIT6</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/STMicroelectronics/STM32H753ZIT6</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -6089,11 +5877,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">511-STM32H753ZIT6</t>
-        </is>
-      </c>
+      <c r="O56"/>
       <c r="P56">
         <v>17.13</v>
       </c>
@@ -6171,7 +5955,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=1043</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Keystone-Electronics/1043</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -6195,11 +5979,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">534-1043</t>
-        </is>
-      </c>
+      <c r="O57"/>
       <c r="P57">
         <v>2.99</v>
       </c>
@@ -6277,7 +6057,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=PTS645SM43SMTR92LFS</t>
+          <t xml:space="preserve">https://www.mouser.com/ProductDetail/CK/PTS645SM43SMTR92LFS</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -6301,11 +6081,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">611-PTS645SM43SMTR92</t>
-        </is>
-      </c>
+      <c r="O58"/>
       <c r="P58">
         <v>0.36</v>
       </c>
@@ -6379,7 +6155,7 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=SRP7028A-4R7M</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/SRP7028A-4R7M</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -6403,11 +6179,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-SRP7028A-4R7M</t>
-        </is>
-      </c>
+      <c r="O59"/>
       <c r="P59">
         <v>1.1</v>
       </c>
@@ -6485,7 +6257,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=RT0603BRD0794K2L</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/YAGEO/RT0603BRD0794K2L</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -6513,11 +6285,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">603-RT0603BRD0794K2L</t>
-        </is>
-      </c>
+      <c r="O60"/>
       <c r="P60">
         <v>0.1</v>
       </c>
@@ -6595,7 +6363,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05C220JB5NNNC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05C220JB5NNNC</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -6619,11 +6387,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL05C220JB5NNNC</t>
-        </is>
-      </c>
+      <c r="O61"/>
       <c r="P61">
         <v>0.1</v>
       </c>
@@ -6701,7 +6465,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05C100JB5NNNC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05C100JB5NNNC</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -6725,11 +6489,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL05C100JB5NNNC</t>
-        </is>
-      </c>
+      <c r="O62"/>
       <c r="P62">
         <v>0.1</v>
       </c>
@@ -6807,7 +6567,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05C750JB5NNNC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05C750JB5NNNC</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -6831,11 +6591,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL05C750JB5NNNC</t>
-        </is>
-      </c>
+      <c r="O63"/>
       <c r="P63">
         <v>0.1</v>
       </c>
@@ -6909,7 +6665,7 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=599-0160-137F</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Dialight/599-0160-137F</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -6933,11 +6689,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">645-599-0160-137F</t>
-        </is>
-      </c>
+      <c r="O64"/>
       <c r="P64">
         <v>0.29</v>
       </c>
@@ -7015,7 +6767,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL31A226KAHNNNE</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL31A226KAHNNNE</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -7039,11 +6791,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL31A226KAHNNNE</t>
-        </is>
-      </c>
+      <c r="O65"/>
       <c r="P65">
         <v>0.38</v>
       </c>
@@ -7121,7 +6869,7 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=TPS2121RUXR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPS2121RUXR</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -7145,11 +6893,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-TPS2121RUXR</t>
-        </is>
-      </c>
+      <c r="O66"/>
       <c r="P66">
         <v>2.44</v>
       </c>
@@ -7227,7 +6971,7 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-6652ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-6652ELF</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -7255,11 +6999,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603-FX6652ELF</t>
-        </is>
-      </c>
+      <c r="O67"/>
       <c r="P67">
         <v>0.1</v>
       </c>
@@ -7337,7 +7077,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=USB4105-GF-A</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/GCT/USB4105-GF-A?qs=KUoIvG%2F9IlY%2FMLlBMpStpA%3D%3D</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -7361,11 +7101,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">640-USB4105-GF-A</t>
-        </is>
-      </c>
+      <c r="O68"/>
       <c r="P68">
         <v>0.93</v>
       </c>
@@ -7443,7 +7179,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL21A475KAQNNNE</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL21A475KAQNNNE</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -7467,11 +7203,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL21A475KAQNNNE</t>
-        </is>
-      </c>
+      <c r="O69"/>
       <c r="P69">
         <v>0.11</v>
       </c>
@@ -7549,7 +7281,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=RC0603FR-07220RL</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/YAGEO/RC0603FR-07220RL</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -7573,11 +7305,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">603-RC0603FR-07220RL</t>
-        </is>
-      </c>
+      <c r="O70"/>
       <c r="P70">
         <v>0.1</v>
       </c>
@@ -7655,7 +7383,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=TPD2E009DBZR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TPD2E009DBZR</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -7679,11 +7407,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-TPD2E009DBZR</t>
-        </is>
-      </c>
+      <c r="O71"/>
       <c r="P71">
         <v>0.79</v>
       </c>
@@ -7761,7 +7485,7 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=150060GS75000</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/150060GS75000</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -7785,11 +7509,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-150060GS75000</t>
-        </is>
-      </c>
+      <c r="O72"/>
       <c r="P72">
         <v>0.16</v>
       </c>
@@ -7867,7 +7587,7 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL05B332KB5NNNC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL05B332KB5NNNC</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -7891,11 +7611,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL05B332KB5NNNC</t>
-        </is>
-      </c>
+      <c r="O73"/>
       <c r="P73">
         <v>0.1</v>
       </c>
@@ -7973,7 +7689,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=SN74AHC1G125DRLR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/SN74AHC1G125DRLR</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -7997,11 +7713,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-SN74AHC1G125DRLR</t>
-        </is>
-      </c>
+      <c r="O74"/>
       <c r="P74">
         <v>0.22</v>
       </c>
@@ -8075,7 +7787,7 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=IC51-0644-807</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Yamaichi-Electronics/IC51-0644-807</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -8099,11 +7811,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">945-IC51-0644-807</t>
-        </is>
-      </c>
+      <c r="O75"/>
       <c r="P75">
         <v>126.53</v>
       </c>
@@ -8181,7 +7889,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=SN74LVC1GU04DRLR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/SN74LVC1GU04DRLR</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -8205,11 +7913,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-SN74LVC1GU04DRLR</t>
-        </is>
-      </c>
+      <c r="O76"/>
       <c r="P76">
         <v>0.36</v>
       </c>
@@ -8287,7 +7991,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL10A475KO8NNNC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL10A475KO8NNNC</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -8311,11 +8015,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL10A475KO8NNNC</t>
-        </is>
-      </c>
+      <c r="O77"/>
       <c r="P77">
         <v>0.12</v>
       </c>
@@ -8393,7 +8093,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=TXS0102DCUR</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Texas-Instruments/TXS0102DCUR</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -8417,11 +8117,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-TXS0102DCUR</t>
-        </is>
-      </c>
+      <c r="O78"/>
       <c r="P78">
         <v>0.63</v>
       </c>
@@ -8499,7 +8195,7 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=AC0603FR-07255KL</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/YAGEO/AC0603FR-07255KL</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -8527,11 +8223,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">603-AC0603FR-07255KL</t>
-        </is>
-      </c>
+      <c r="O79"/>
       <c r="P79">
         <v>0.1</v>
       </c>
@@ -8609,7 +8301,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW06035K05FKEA</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW06035K05FKEA</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -8637,11 +8329,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">71-CRCW0603-5.05K-E3</t>
-        </is>
-      </c>
+      <c r="O80"/>
       <c r="P80">
         <v>0.1</v>
       </c>
@@ -8719,7 +8407,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=JS102011SAQN</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/CK/JS102011SAQN</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -8743,11 +8431,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">611-JS102011SAQN</t>
-        </is>
-      </c>
+      <c r="O81"/>
       <c r="P81">
         <v>0.84</v>
       </c>
@@ -8825,7 +8509,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=KTR03EZPF3403</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/ROHM-Semiconductor/KTR03EZPF3403</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -8853,11 +8537,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">755-KTR03EZPF3403</t>
-        </is>
-      </c>
+      <c r="O82"/>
       <c r="P82">
         <v>0.19</v>
       </c>
@@ -8935,7 +8615,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CRCW06033R32FKTA</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Vishay/CRCW06033R32FKTA</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -8963,11 +8643,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">71-CRCW0603-3.32</t>
-        </is>
-      </c>
+      <c r="O83"/>
       <c r="P83">
         <v>0.29</v>
       </c>
@@ -9045,7 +8721,7 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CR0603-FX-6800ELF</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Bourns/CR0603-FX-6800ELF</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -9073,11 +8749,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">652-CR0603FX-6800ELF</t>
-        </is>
-      </c>
+      <c r="O84"/>
       <c r="P84">
         <v>0.1</v>
       </c>
@@ -9155,7 +8827,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=742792022</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/742792022</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -9179,11 +8851,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-742792022</t>
-        </is>
-      </c>
+      <c r="O85"/>
       <c r="P85">
         <v>0.16</v>
       </c>
@@ -9261,7 +8929,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=560112116151</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Wurth-Elektronik/560112116151</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -9289,11 +8957,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-560112116151</t>
-        </is>
-      </c>
+      <c r="O86"/>
       <c r="P86">
         <v>0.11</v>
       </c>
@@ -9371,7 +9035,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=ERJ-PA2F1242X</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Panasonic/ERJ-PA2F1242X</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -9399,11 +9063,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">667-ERJ-PA2F1242X</t>
-        </is>
-      </c>
+      <c r="O87"/>
       <c r="P87">
         <v>0.28</v>
       </c>
@@ -9481,7 +9141,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=QSH-060-01-H-D-A</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samtec/QSH-060-01-H-D-A</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -9505,11 +9165,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O88" t="inlineStr">
-        <is>
-          <t xml:space="preserve">200-QSH06001HDA</t>
-        </is>
-      </c>
+      <c r="O88"/>
       <c r="P88">
         <v>22.49</v>
       </c>
@@ -9587,7 +9243,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.mouser.com/c/?q=CL10A105KB8NNNC</t>
+          <t xml:space="preserve">https://www.mouser.com/en/ProductDetail/Samsung-Electro-Mechanics/CL10A105KB8NNNC</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -9611,11 +9267,7 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">187-CL10A105KB8NNNC</t>
-        </is>
-      </c>
+      <c r="O89"/>
       <c r="P89">
         <v>0.11</v>
       </c>

</xml_diff>

<commit_message>
Fill every FINALE SAUCE record with real distributor data (54 direct + 34 via Firecrawl), all 88 keyed to the owner's verbatim links
</commit_message>
<xml_diff>
--- a/docs/FINALE_SAUCE_BOM.xlsx
+++ b/docs/FINALE_SAUCE_BOM.xlsx
@@ -74,7 +74,7 @@
     <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="11" customWidth="1"/>
     <col min="18" max="18" width="9" customWidth="1"/>
-    <col min="19" max="19" width="11" customWidth="1"/>
+    <col min="19" max="19" width="13" customWidth="1"/>
     <col min="20" max="20" width="9" customWidth="1"/>
     <col min="21" max="21" width="11" customWidth="1"/>
     <col min="22" max="22" width="17" customWidth="1"/>
@@ -839,7 +839,7 @@
         <v>0.6</v>
       </c>
       <c r="R7">
-        <v>52599</v>
+        <v>52594</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         <v>0.2</v>
       </c>
       <c r="R8">
-        <v>1496328</v>
+        <v>1496308</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
         <v>1.09</v>
       </c>
       <c r="R10">
-        <v>526042</v>
+        <v>525994</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philippines</t>
+          <t xml:space="preserve">Japan</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1475,14 +1475,20 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O13"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">81-GCM1555C1HR75CA6J</t>
+        </is>
+      </c>
       <c r="P13">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="Q13">
-        <v>0.1</v>
-      </c>
-      <c r="R13"/>
+        <v>0.15</v>
+      </c>
+      <c r="R13">
+        <v>35585</v>
+      </c>
       <c r="S13" t="inlineStr">
         <is>
           <t xml:space="preserve">Active</t>
@@ -1492,20 +1498,22 @@
         <v>1</v>
       </c>
       <c r="U13">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="V13">
-        <v>0.021</v>
+        <v>0.15</v>
       </c>
       <c r="W13">
-        <v>0.21</v>
-      </c>
-      <c r="X13"/>
+        <v>0.45</v>
+      </c>
+      <c r="X13">
+        <v>0</v>
+      </c>
       <c r="Y13">
         <v>0</v>
       </c>
       <c r="Z13">
-        <v>0.21</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="14">
@@ -1809,7 +1817,7 @@
         <v>0.1</v>
       </c>
       <c r="R16">
-        <v>874450</v>
+        <v>874350</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -2021,7 +2029,7 @@
         <v>3.12</v>
       </c>
       <c r="R18">
-        <v>21510</v>
+        <v>21500</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -2783,7 +2791,7 @@
         <v>0.93</v>
       </c>
       <c r="R25">
-        <v>481287</v>
+        <v>481266</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
@@ -2881,15 +2889,19 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O26"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">187-CL31A226MAHNNNE</t>
+        </is>
+      </c>
       <c r="P26">
-        <v>0.38</v>
+        <v>0.65</v>
       </c>
       <c r="Q26">
-        <v>3.04</v>
+        <v>5.2</v>
       </c>
       <c r="R26">
-        <v>0</v>
+        <v>12611</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
@@ -2903,19 +2915,19 @@
         <v>24</v>
       </c>
       <c r="V26">
-        <v>0.166</v>
+        <v>0.431</v>
       </c>
       <c r="W26">
-        <v>3.984</v>
+        <v>10.344</v>
       </c>
       <c r="X26">
-        <v>7.89</v>
+        <v>8</v>
       </c>
       <c r="Y26">
-        <v>0.3143</v>
+        <v>0.8275</v>
       </c>
       <c r="Z26">
-        <v>4.2983</v>
+        <v>11.1715</v>
       </c>
     </row>
     <row r="27">
@@ -2999,7 +3011,7 @@
         <v>7.82</v>
       </c>
       <c r="R27">
-        <v>58284</v>
+        <v>58274</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
@@ -3325,7 +3337,7 @@
         <v>1.43</v>
       </c>
       <c r="R30">
-        <v>47115</v>
+        <v>47090</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -3533,7 +3545,7 @@
         <v>0.8</v>
       </c>
       <c r="R32">
-        <v>64742</v>
+        <v>64322</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
@@ -4165,7 +4177,7 @@
         <v>0.22</v>
       </c>
       <c r="R38">
-        <v>189</v>
+        <v>0</v>
       </c>
       <c r="S38" t="inlineStr">
         <is>
@@ -5143,7 +5155,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active</t>
+          <t xml:space="preserve">New Product</t>
         </is>
       </c>
       <c r="T47">
@@ -5567,7 +5579,7 @@
         <v>0.16</v>
       </c>
       <c r="R51">
-        <v>368610</v>
+        <v>368302</v>
       </c>
       <c r="S51" t="inlineStr">
         <is>
@@ -5779,7 +5791,7 @@
         <v>2.99</v>
       </c>
       <c r="R53">
-        <v>9773</v>
+        <v>9743</v>
       </c>
       <c r="S53" t="inlineStr">
         <is>
@@ -5987,15 +5999,19 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O55"/>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">187-CL05C100JB5NNWC</t>
+        </is>
+      </c>
       <c r="P55">
-        <v>0.1</v>
+        <v>0.23</v>
       </c>
       <c r="Q55">
-        <v>0.3</v>
+        <v>0.69</v>
       </c>
       <c r="R55">
-        <v>118171</v>
+        <v>99958</v>
       </c>
       <c r="S55" t="inlineStr">
         <is>
@@ -6009,19 +6025,19 @@
         <v>10</v>
       </c>
       <c r="V55">
-        <v>0.019</v>
+        <v>0.081</v>
       </c>
       <c r="W55">
-        <v>0.19</v>
+        <v>0.81</v>
       </c>
       <c r="X55">
-        <v>8</v>
+        <v>7.83</v>
       </c>
       <c r="Y55">
-        <v>0.0152</v>
+        <v>0.0634</v>
       </c>
       <c r="Z55">
-        <v>0.2052</v>
+        <v>0.8734</v>
       </c>
     </row>
     <row r="56">
@@ -6321,7 +6337,7 @@
         <v>11.5</v>
       </c>
       <c r="R58">
-        <v>5176</v>
+        <v>4882</v>
       </c>
       <c r="S58" t="inlineStr">
         <is>
@@ -6643,7 +6659,7 @@
         <v>2.44</v>
       </c>
       <c r="R61">
-        <v>16194</v>
+        <v>14155</v>
       </c>
       <c r="S61" t="inlineStr">
         <is>
@@ -6753,7 +6769,7 @@
         <v>0.1</v>
       </c>
       <c r="R62">
-        <v>331735</v>
+        <v>331725</v>
       </c>
       <c r="S62" t="inlineStr">
         <is>
@@ -6843,7 +6859,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philippines</t>
+          <t xml:space="preserve">China</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -6851,7 +6867,11 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O63"/>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">187-CL05B332KB5NNWC</t>
+        </is>
+      </c>
       <c r="P63">
         <v>0.1</v>
       </c>
@@ -6859,7 +6879,7 @@
         <v>0.1</v>
       </c>
       <c r="R63">
-        <v>125342</v>
+        <v>80721</v>
       </c>
       <c r="S63" t="inlineStr">
         <is>
@@ -6873,19 +6893,19 @@
         <v>10</v>
       </c>
       <c r="V63">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="W63">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="X63">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Y63">
-        <v>0.0096</v>
+        <v>0.013</v>
       </c>
       <c r="Z63">
-        <v>0.1296</v>
+        <v>0.143</v>
       </c>
     </row>
     <row r="64">
@@ -6969,7 +6989,7 @@
         <v>0.1</v>
       </c>
       <c r="R64">
-        <v>6976557</v>
+        <v>6731048</v>
       </c>
       <c r="S64" t="inlineStr">
         <is>
@@ -7185,7 +7205,7 @@
         <v>0.79</v>
       </c>
       <c r="R66">
-        <v>10330</v>
+        <v>4367</v>
       </c>
       <c r="S66" t="inlineStr">
         <is>
@@ -7291,7 +7311,7 @@
         <v>6.99</v>
       </c>
       <c r="R67">
-        <v>3754</v>
+        <v>3744</v>
       </c>
       <c r="S67" t="inlineStr">
         <is>
@@ -7617,7 +7637,7 @@
         <v>0.16</v>
       </c>
       <c r="R70">
-        <v>146494</v>
+        <v>146444</v>
       </c>
       <c r="S70" t="inlineStr">
         <is>
@@ -8269,7 +8289,7 @@
         <v>0.12</v>
       </c>
       <c r="R76">
-        <v>389441</v>
+        <v>385121</v>
       </c>
       <c r="S76" t="inlineStr">
         <is>
@@ -8481,7 +8501,7 @@
         <v>1.26</v>
       </c>
       <c r="R78">
-        <v>111487</v>
+        <v>111475</v>
       </c>
       <c r="S78" t="inlineStr">
         <is>
@@ -9121,14 +9141,20 @@
           <t xml:space="preserve">Mouser</t>
         </is>
       </c>
-      <c r="O84"/>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">611-PTS645SK43SMTR92</t>
+        </is>
+      </c>
       <c r="P84">
         <v>0.36</v>
       </c>
       <c r="Q84">
         <v>0.72</v>
       </c>
-      <c r="R84"/>
+      <c r="R84">
+        <v>87087</v>
+      </c>
       <c r="S84" t="inlineStr">
         <is>
           <t xml:space="preserve">Active</t>
@@ -9146,12 +9172,14 @@
       <c r="W84">
         <v>2.16</v>
       </c>
-      <c r="X84"/>
+      <c r="X84">
+        <v>8.06</v>
+      </c>
       <c r="Y84">
-        <v>0</v>
+        <v>0.1741</v>
       </c>
       <c r="Z84">
-        <v>2.16</v>
+        <v>2.3341</v>
       </c>
     </row>
     <row r="85">
@@ -9345,7 +9373,7 @@
         <v>0.48</v>
       </c>
       <c r="R86">
-        <v>18238</v>
+        <v>18188</v>
       </c>
       <c r="S86" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
BOM xlsx: emit live formulas for the cost columns and the TOTAL row (recalc on open), and set Min Qty to the per-board quantity
</commit_message>
<xml_diff>
--- a/docs/FINALE_SAUCE_BOM.xlsx
+++ b/docs/FINALE_SAUCE_BOM.xlsx
@@ -4,6 +4,7 @@
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -299,6 +300,7 @@
         <v>0.1</v>
       </c>
       <c r="Q2" s="3">
+        <f>P2*B2</f>
         <v>0.1</v>
       </c>
       <c r="R2">
@@ -319,15 +321,18 @@
         <v>0.016</v>
       </c>
       <c r="W2" s="3">
+        <f>V2*U2</f>
         <v>0.16</v>
       </c>
       <c r="X2">
         <v>0</v>
       </c>
       <c r="Y2" s="3">
+        <f>W2*X2/100</f>
         <v>0</v>
       </c>
       <c r="Z2" s="3">
+        <f>W2+Y2</f>
         <v>0.16</v>
       </c>
     </row>
@@ -409,6 +414,7 @@
         <v>0.11</v>
       </c>
       <c r="Q3" s="3">
+        <f>P3*B3</f>
         <v>0.44</v>
       </c>
       <c r="R3">
@@ -420,7 +426,7 @@
         </is>
       </c>
       <c r="T3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U3">
         <v>12</v>
@@ -429,15 +435,18 @@
         <v>0.102</v>
       </c>
       <c r="W3" s="3">
+        <f>V3*U3</f>
         <v>1.224</v>
       </c>
       <c r="X3">
         <v>0</v>
       </c>
       <c r="Y3" s="3">
+        <f>W3*X3/100</f>
         <v>0</v>
       </c>
       <c r="Z3" s="3">
+        <f>W3+Y3</f>
         <v>1.224</v>
       </c>
     </row>
@@ -519,6 +528,7 @@
         <v>0.1</v>
       </c>
       <c r="Q4" s="3">
+        <f>P4*B4</f>
         <v>6</v>
       </c>
       <c r="R4">
@@ -530,7 +540,7 @@
         </is>
       </c>
       <c r="T4">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="U4">
         <v>180</v>
@@ -539,15 +549,18 @@
         <v>0.01</v>
       </c>
       <c r="W4" s="3">
+        <f>V4*U4</f>
         <v>1.8</v>
       </c>
       <c r="X4">
         <v>8</v>
       </c>
       <c r="Y4" s="3">
+        <f>W4*X4/100</f>
         <v>0.144</v>
       </c>
       <c r="Z4" s="3">
+        <f>W4+Y4</f>
         <v>1.944</v>
       </c>
     </row>
@@ -629,6 +642,7 @@
         <v>0.1</v>
       </c>
       <c r="Q5" s="3">
+        <f>P5*B5</f>
         <v>0.1</v>
       </c>
       <c r="R5">
@@ -649,15 +663,18 @@
         <v>0.025</v>
       </c>
       <c r="W5" s="3">
+        <f>V5*U5</f>
         <v>0.25</v>
       </c>
       <c r="X5">
         <v>10</v>
       </c>
       <c r="Y5" s="3">
+        <f>W5*X5/100</f>
         <v>0.025</v>
       </c>
       <c r="Z5" s="3">
+        <f>W5+Y5</f>
         <v>0.275</v>
       </c>
     </row>
@@ -735,6 +752,7 @@
         <v>0.14</v>
       </c>
       <c r="Q6" s="3">
+        <f>P6*B6</f>
         <v>0.56</v>
       </c>
       <c r="R6">
@@ -746,7 +764,7 @@
         </is>
       </c>
       <c r="T6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U6">
         <v>12</v>
@@ -755,15 +773,18 @@
         <v>0.092</v>
       </c>
       <c r="W6" s="3">
+        <f>V6*U6</f>
         <v>1.104</v>
       </c>
       <c r="X6">
         <v>37.86</v>
       </c>
       <c r="Y6" s="3">
+        <f>W6*X6/100</f>
         <v>0.418</v>
       </c>
       <c r="Z6" s="3">
+        <f>W6+Y6</f>
         <v>1.522</v>
       </c>
     </row>
@@ -841,6 +862,7 @@
         <v>0.6</v>
       </c>
       <c r="Q7" s="3">
+        <f>P7*B7</f>
         <v>0.6</v>
       </c>
       <c r="R7">
@@ -861,15 +883,18 @@
         <v>0.6</v>
       </c>
       <c r="W7" s="3">
+        <f>V7*U7</f>
         <v>1.8</v>
       </c>
       <c r="X7">
         <v>8</v>
       </c>
       <c r="Y7" s="3">
+        <f>W7*X7/100</f>
         <v>0.144</v>
       </c>
       <c r="Z7" s="3">
+        <f>W7+Y7</f>
         <v>1.944</v>
       </c>
     </row>
@@ -951,6 +976,7 @@
         <v>0.1</v>
       </c>
       <c r="Q8" s="3">
+        <f>P8*B8</f>
         <v>0.2</v>
       </c>
       <c r="R8">
@@ -962,7 +988,7 @@
         </is>
       </c>
       <c r="T8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U8">
         <v>10</v>
@@ -971,15 +997,18 @@
         <v>0.012</v>
       </c>
       <c r="W8" s="3">
+        <f>V8*U8</f>
         <v>0.12</v>
       </c>
       <c r="X8">
         <v>0</v>
       </c>
       <c r="Y8" s="3">
+        <f>W8*X8/100</f>
         <v>0</v>
       </c>
       <c r="Z8" s="3">
+        <f>W8+Y8</f>
         <v>0.12</v>
       </c>
     </row>
@@ -1057,6 +1086,7 @@
         <v>0.52</v>
       </c>
       <c r="Q9" s="3">
+        <f>P9*B9</f>
         <v>3.64</v>
       </c>
       <c r="R9">
@@ -1068,7 +1098,7 @@
         </is>
       </c>
       <c r="T9">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="U9">
         <v>21</v>
@@ -1077,15 +1107,18 @@
         <v>0.367</v>
       </c>
       <c r="W9" s="3">
+        <f>V9*U9</f>
         <v>7.707</v>
       </c>
       <c r="X9">
         <v>0</v>
       </c>
       <c r="Y9" s="3">
+        <f>W9*X9/100</f>
         <v>0</v>
       </c>
       <c r="Z9" s="3">
+        <f>W9+Y9</f>
         <v>7.707</v>
       </c>
     </row>
@@ -1163,6 +1196,7 @@
         <v>1.09</v>
       </c>
       <c r="Q10" s="3">
+        <f>P10*B10</f>
         <v>1.09</v>
       </c>
       <c r="R10">
@@ -1183,15 +1217,18 @@
         <v>1.09</v>
       </c>
       <c r="W10" s="3">
+        <f>V10*U10</f>
         <v>3.27</v>
       </c>
       <c r="X10">
         <v>7.98</v>
       </c>
       <c r="Y10" s="3">
+        <f>W10*X10/100</f>
         <v>0.2609</v>
       </c>
       <c r="Z10" s="3">
+        <f>W10+Y10</f>
         <v>3.5309</v>
       </c>
     </row>
@@ -1273,6 +1310,7 @@
         <v>0.46</v>
       </c>
       <c r="Q11" s="3">
+        <f>P11*B11</f>
         <v>2.3</v>
       </c>
       <c r="R11">
@@ -1284,7 +1322,7 @@
         </is>
       </c>
       <c r="T11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U11">
         <v>15</v>
@@ -1293,15 +1331,18 @@
         <v>0.306</v>
       </c>
       <c r="W11" s="3">
+        <f>V11*U11</f>
         <v>4.59</v>
       </c>
       <c r="X11">
         <v>8.04</v>
       </c>
       <c r="Y11" s="3">
+        <f>W11*X11/100</f>
         <v>0.369</v>
       </c>
       <c r="Z11" s="3">
+        <f>W11+Y11</f>
         <v>4.959</v>
       </c>
     </row>
@@ -1379,6 +1420,7 @@
         <v>3.19</v>
       </c>
       <c r="Q12" s="3">
+        <f>P12*B12</f>
         <v>3.19</v>
       </c>
       <c r="R12">
@@ -1399,15 +1441,18 @@
         <v>3.19</v>
       </c>
       <c r="W12" s="3">
+        <f>V12*U12</f>
         <v>9.57</v>
       </c>
       <c r="X12">
         <v>37.93</v>
       </c>
       <c r="Y12" s="3">
+        <f>W12*X12/100</f>
         <v>3.6299</v>
       </c>
       <c r="Z12" s="3">
+        <f>W12+Y12</f>
         <v>13.1999</v>
       </c>
     </row>
@@ -1489,6 +1534,7 @@
         <v>0.15</v>
       </c>
       <c r="Q13" s="3">
+        <f>P13*B13</f>
         <v>0.15</v>
       </c>
       <c r="R13">
@@ -1509,15 +1555,18 @@
         <v>0.15</v>
       </c>
       <c r="W13" s="3">
+        <f>V13*U13</f>
         <v>0.45</v>
       </c>
       <c r="X13">
         <v>0</v>
       </c>
       <c r="Y13" s="3">
+        <f>W13*X13/100</f>
         <v>0</v>
       </c>
       <c r="Z13" s="3">
+        <f>W13+Y13</f>
         <v>0.45</v>
       </c>
     </row>
@@ -1599,6 +1648,7 @@
         <v>0.11</v>
       </c>
       <c r="Q14" s="3">
+        <f>P14*B14</f>
         <v>0.88</v>
       </c>
       <c r="R14">
@@ -1610,7 +1660,7 @@
         </is>
       </c>
       <c r="T14">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="U14">
         <v>24</v>
@@ -1619,15 +1669,18 @@
         <v>0.102</v>
       </c>
       <c r="W14" s="3">
+        <f>V14*U14</f>
         <v>2.448</v>
       </c>
       <c r="X14">
         <v>0</v>
       </c>
       <c r="Y14" s="3">
+        <f>W14*X14/100</f>
         <v>0</v>
       </c>
       <c r="Z14" s="3">
+        <f>W14+Y14</f>
         <v>2.448</v>
       </c>
     </row>
@@ -1709,6 +1762,7 @@
         <v>0.1</v>
       </c>
       <c r="Q15" s="3">
+        <f>P15*B15</f>
         <v>0.4</v>
       </c>
       <c r="R15">
@@ -1720,7 +1774,7 @@
         </is>
       </c>
       <c r="T15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U15">
         <v>12</v>
@@ -1729,15 +1783,18 @@
         <v>0.033</v>
       </c>
       <c r="W15" s="3">
+        <f>V15*U15</f>
         <v>0.396</v>
       </c>
       <c r="X15">
         <v>8</v>
       </c>
       <c r="Y15" s="3">
+        <f>W15*X15/100</f>
         <v>0.0317</v>
       </c>
       <c r="Z15" s="3">
+        <f>W15+Y15</f>
         <v>0.4277</v>
       </c>
     </row>
@@ -1819,6 +1876,7 @@
         <v>0.1</v>
       </c>
       <c r="Q16" s="3">
+        <f>P16*B16</f>
         <v>0.1</v>
       </c>
       <c r="R16">
@@ -1839,15 +1897,18 @@
         <v>0.012</v>
       </c>
       <c r="W16" s="3">
+        <f>V16*U16</f>
         <v>0.12</v>
       </c>
       <c r="X16">
         <v>0</v>
       </c>
       <c r="Y16" s="3">
+        <f>W16*X16/100</f>
         <v>0</v>
       </c>
       <c r="Z16" s="3">
+        <f>W16+Y16</f>
         <v>0.12</v>
       </c>
     </row>
@@ -1925,6 +1986,7 @@
         <v>2.73</v>
       </c>
       <c r="Q17" s="3">
+        <f>P17*B17</f>
         <v>2.73</v>
       </c>
       <c r="R17">
@@ -1945,15 +2007,18 @@
         <v>2.73</v>
       </c>
       <c r="W17" s="3">
+        <f>V17*U17</f>
         <v>8.19</v>
       </c>
       <c r="X17">
         <v>0</v>
       </c>
       <c r="Y17" s="3">
+        <f>W17*X17/100</f>
         <v>0</v>
       </c>
       <c r="Z17" s="3">
+        <f>W17+Y17</f>
         <v>8.19</v>
       </c>
     </row>
@@ -2027,6 +2092,7 @@
         <v>0.39</v>
       </c>
       <c r="Q18" s="3">
+        <f>P18*B18</f>
         <v>3.12</v>
       </c>
       <c r="R18">
@@ -2038,7 +2104,7 @@
         </is>
       </c>
       <c r="T18">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="U18">
         <v>25</v>
@@ -2047,15 +2113,18 @@
         <v>0.28</v>
       </c>
       <c r="W18" s="3">
+        <f>V18*U18</f>
         <v>7</v>
       </c>
       <c r="X18">
         <v>0</v>
       </c>
       <c r="Y18" s="3">
+        <f>W18*X18/100</f>
         <v>0</v>
       </c>
       <c r="Z18" s="3">
+        <f>W18+Y18</f>
         <v>7</v>
       </c>
     </row>
@@ -2137,6 +2206,7 @@
         <v>0.1</v>
       </c>
       <c r="Q19" s="3">
+        <f>P19*B19</f>
         <v>0.2</v>
       </c>
       <c r="R19">
@@ -2148,7 +2218,7 @@
         </is>
       </c>
       <c r="T19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U19">
         <v>10</v>
@@ -2157,15 +2227,18 @@
         <v>0.015</v>
       </c>
       <c r="W19" s="3">
+        <f>V19*U19</f>
         <v>0.15</v>
       </c>
       <c r="X19">
         <v>8</v>
       </c>
       <c r="Y19" s="3">
+        <f>W19*X19/100</f>
         <v>0.012</v>
       </c>
       <c r="Z19" s="3">
+        <f>W19+Y19</f>
         <v>0.162</v>
       </c>
     </row>
@@ -2247,6 +2320,7 @@
         <v>0.31</v>
       </c>
       <c r="Q20" s="3">
+        <f>P20*B20</f>
         <v>0.31</v>
       </c>
       <c r="R20">
@@ -2267,15 +2341,18 @@
         <v>0.31</v>
       </c>
       <c r="W20" s="3">
+        <f>V20*U20</f>
         <v>0.93</v>
       </c>
       <c r="X20">
         <v>0</v>
       </c>
       <c r="Y20" s="3">
+        <f>W20*X20/100</f>
         <v>0</v>
       </c>
       <c r="Z20" s="3">
+        <f>W20+Y20</f>
         <v>0.93</v>
       </c>
     </row>
@@ -2357,6 +2434,7 @@
         <v>0.25</v>
       </c>
       <c r="Q21" s="3">
+        <f>P21*B21</f>
         <v>0.25</v>
       </c>
       <c r="R21">
@@ -2377,15 +2455,18 @@
         <v>0.063</v>
       </c>
       <c r="W21" s="3">
+        <f>V21*U21</f>
         <v>0.63</v>
       </c>
       <c r="X21">
         <v>0</v>
       </c>
       <c r="Y21" s="3">
+        <f>W21*X21/100</f>
         <v>0</v>
       </c>
       <c r="Z21" s="3">
+        <f>W21+Y21</f>
         <v>0.63</v>
       </c>
     </row>
@@ -2463,6 +2544,7 @@
         <v>1.68</v>
       </c>
       <c r="Q22" s="3">
+        <f>P22*B22</f>
         <v>1.68</v>
       </c>
       <c r="R22">
@@ -2483,15 +2565,18 @@
         <v>1.68</v>
       </c>
       <c r="W22" s="3">
+        <f>V22*U22</f>
         <v>5.04</v>
       </c>
       <c r="X22">
         <v>0</v>
       </c>
       <c r="Y22" s="3">
+        <f>W22*X22/100</f>
         <v>0</v>
       </c>
       <c r="Z22" s="3">
+        <f>W22+Y22</f>
         <v>5.04</v>
       </c>
     </row>
@@ -2573,6 +2658,7 @@
         <v>0.13</v>
       </c>
       <c r="Q23" s="3">
+        <f>P23*B23</f>
         <v>0.13</v>
       </c>
       <c r="R23">
@@ -2593,15 +2679,18 @@
         <v>0.033</v>
       </c>
       <c r="W23" s="3">
+        <f>V23*U23</f>
         <v>0.33</v>
       </c>
       <c r="X23">
         <v>0</v>
       </c>
       <c r="Y23" s="3">
+        <f>W23*X23/100</f>
         <v>0</v>
       </c>
       <c r="Z23" s="3">
+        <f>W23+Y23</f>
         <v>0.33</v>
       </c>
     </row>
@@ -2683,6 +2772,7 @@
         <v>0.31</v>
       </c>
       <c r="Q24" s="3">
+        <f>P24*B24</f>
         <v>0.62</v>
       </c>
       <c r="R24">
@@ -2694,7 +2784,7 @@
         </is>
       </c>
       <c r="T24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U24">
         <v>10</v>
@@ -2703,15 +2793,18 @@
         <v>0.135</v>
       </c>
       <c r="W24" s="3">
+        <f>V24*U24</f>
         <v>1.35</v>
       </c>
       <c r="X24">
         <v>10</v>
       </c>
       <c r="Y24" s="3">
+        <f>W24*X24/100</f>
         <v>0.135</v>
       </c>
       <c r="Z24" s="3">
+        <f>W24+Y24</f>
         <v>1.485</v>
       </c>
     </row>
@@ -2789,6 +2882,7 @@
         <v>0.76</v>
       </c>
       <c r="Q25" s="3">
+        <f>P25*B25</f>
         <v>1.52</v>
       </c>
       <c r="R25">
@@ -2800,7 +2894,7 @@
         </is>
       </c>
       <c r="T25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U25">
         <v>6</v>
@@ -2809,15 +2903,18 @@
         <v>0.76</v>
       </c>
       <c r="W25" s="3">
+        <f>V25*U25</f>
         <v>4.56</v>
       </c>
       <c r="X25">
         <v>0</v>
       </c>
       <c r="Y25" s="3">
+        <f>W25*X25/100</f>
         <v>0</v>
       </c>
       <c r="Z25" s="3">
+        <f>W25+Y25</f>
         <v>4.56</v>
       </c>
     </row>
@@ -2895,6 +2992,7 @@
         <v>0.93</v>
       </c>
       <c r="Q26" s="3">
+        <f>P26*B26</f>
         <v>0.93</v>
       </c>
       <c r="R26">
@@ -2915,15 +3013,18 @@
         <v>0.93</v>
       </c>
       <c r="W26" s="3">
+        <f>V26*U26</f>
         <v>2.79</v>
       </c>
       <c r="X26">
         <v>30</v>
       </c>
       <c r="Y26" s="3">
+        <f>W26*X26/100</f>
         <v>0.837</v>
       </c>
       <c r="Z26" s="3">
+        <f>W26+Y26</f>
         <v>3.627</v>
       </c>
     </row>
@@ -3005,6 +3106,7 @@
         <v>0.65</v>
       </c>
       <c r="Q27" s="3">
+        <f>P27*B27</f>
         <v>5.2</v>
       </c>
       <c r="R27">
@@ -3016,7 +3118,7 @@
         </is>
       </c>
       <c r="T27">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="U27">
         <v>24</v>
@@ -3025,15 +3127,18 @@
         <v>0.431</v>
       </c>
       <c r="W27" s="3">
+        <f>V27*U27</f>
         <v>10.344</v>
       </c>
       <c r="X27">
         <v>8</v>
       </c>
       <c r="Y27" s="3">
+        <f>W27*X27/100</f>
         <v>0.8275</v>
       </c>
       <c r="Z27" s="3">
+        <f>W27+Y27</f>
         <v>11.1715</v>
       </c>
     </row>
@@ -3115,6 +3220,7 @@
         <v>0.23</v>
       </c>
       <c r="Q28" s="3">
+        <f>P28*B28</f>
         <v>7.82</v>
       </c>
       <c r="R28">
@@ -3126,7 +3232,7 @@
         </is>
       </c>
       <c r="T28">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="U28">
         <v>102</v>
@@ -3135,15 +3241,18 @@
         <v>0.072</v>
       </c>
       <c r="W28" s="3">
+        <f>V28*U28</f>
         <v>7.344</v>
       </c>
       <c r="X28">
         <v>0</v>
       </c>
       <c r="Y28" s="3">
+        <f>W28*X28/100</f>
         <v>0</v>
       </c>
       <c r="Z28" s="3">
+        <f>W28+Y28</f>
         <v>7.344</v>
       </c>
     </row>
@@ -3221,6 +3330,7 @@
         <v>4.05</v>
       </c>
       <c r="Q29" s="3">
+        <f>P29*B29</f>
         <v>4.05</v>
       </c>
       <c r="R29">
@@ -3241,15 +3351,18 @@
         <v>4.05</v>
       </c>
       <c r="W29" s="3">
+        <f>V29*U29</f>
         <v>12.15</v>
       </c>
       <c r="X29">
         <v>35.06</v>
       </c>
       <c r="Y29" s="3">
+        <f>W29*X29/100</f>
         <v>4.2598</v>
       </c>
       <c r="Z29" s="3">
+        <f>W29+Y29</f>
         <v>16.4098</v>
       </c>
     </row>
@@ -3331,6 +3444,7 @@
         <v>0.13</v>
       </c>
       <c r="Q30" s="3">
+        <f>P30*B30</f>
         <v>0.13</v>
       </c>
       <c r="R30">
@@ -3351,15 +3465,18 @@
         <v>0.033</v>
       </c>
       <c r="W30" s="3">
+        <f>V30*U30</f>
         <v>0.33</v>
       </c>
       <c r="X30">
         <v>0</v>
       </c>
       <c r="Y30" s="3">
+        <f>W30*X30/100</f>
         <v>0</v>
       </c>
       <c r="Z30" s="3">
+        <f>W30+Y30</f>
         <v>0.33</v>
       </c>
     </row>
@@ -3437,6 +3554,7 @@
         <v>1.43</v>
       </c>
       <c r="Q31" s="3">
+        <f>P31*B31</f>
         <v>1.43</v>
       </c>
       <c r="R31">
@@ -3457,15 +3575,18 @@
         <v>1.43</v>
       </c>
       <c r="W31" s="3">
+        <f>V31*U31</f>
         <v>4.29</v>
       </c>
       <c r="X31">
         <v>0</v>
       </c>
       <c r="Y31" s="3">
+        <f>W31*X31/100</f>
         <v>0</v>
       </c>
       <c r="Z31" s="3">
+        <f>W31+Y31</f>
         <v>4.29</v>
       </c>
     </row>
@@ -3539,6 +3660,7 @@
         <v>126.53</v>
       </c>
       <c r="Q32" s="3">
+        <f>P32*B32</f>
         <v>126.53</v>
       </c>
       <c r="R32">
@@ -3559,15 +3681,18 @@
         <v>126.53</v>
       </c>
       <c r="W32" s="3">
+        <f>V32*U32</f>
         <v>379.59</v>
       </c>
       <c r="X32">
         <v>8</v>
       </c>
       <c r="Y32" s="3">
+        <f>W32*X32/100</f>
         <v>30.3672</v>
       </c>
       <c r="Z32" s="3">
+        <f>W32+Y32</f>
         <v>409.9572</v>
       </c>
     </row>
@@ -3645,6 +3770,7 @@
         <v>0.16</v>
       </c>
       <c r="Q33" s="3">
+        <f>P33*B33</f>
         <v>0.8</v>
       </c>
       <c r="R33">
@@ -3656,7 +3782,7 @@
         </is>
       </c>
       <c r="T33">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U33">
         <v>15</v>
@@ -3665,15 +3791,18 @@
         <v>0.101</v>
       </c>
       <c r="W33" s="3">
+        <f>V33*U33</f>
         <v>1.515</v>
       </c>
       <c r="X33">
         <v>0</v>
       </c>
       <c r="Y33" s="3">
+        <f>W33*X33/100</f>
         <v>0</v>
       </c>
       <c r="Z33" s="3">
+        <f>W33+Y33</f>
         <v>1.515</v>
       </c>
     </row>
@@ -3747,6 +3876,7 @@
         <v>0.71</v>
       </c>
       <c r="Q34" s="3">
+        <f>P34*B34</f>
         <v>0.71</v>
       </c>
       <c r="R34">
@@ -3767,15 +3897,18 @@
         <v>0.71</v>
       </c>
       <c r="W34" s="3">
+        <f>V34*U34</f>
         <v>2.13</v>
       </c>
       <c r="X34">
         <v>30</v>
       </c>
       <c r="Y34" s="3">
+        <f>W34*X34/100</f>
         <v>0.639</v>
       </c>
       <c r="Z34" s="3">
+        <f>W34+Y34</f>
         <v>2.769</v>
       </c>
     </row>
@@ -3845,6 +3978,7 @@
         <v>19.95</v>
       </c>
       <c r="Q35" s="3">
+        <f>P35*B35</f>
         <v>19.95</v>
       </c>
       <c r="R35"/>
@@ -3863,6 +3997,7 @@
         <v>19.95</v>
       </c>
       <c r="W35" s="3">
+        <f>V35*U35</f>
         <v>59.85</v>
       </c>
       <c r="X35"/>
@@ -3870,6 +4005,7 @@
         <v>0</v>
       </c>
       <c r="Z35" s="3">
+        <f>W35+Y35</f>
         <v>59.85</v>
       </c>
     </row>
@@ -3943,6 +4079,7 @@
         <v>22.49</v>
       </c>
       <c r="Q36" s="3">
+        <f>P36*B36</f>
         <v>44.98</v>
       </c>
       <c r="R36">
@@ -3954,7 +4091,7 @@
         </is>
       </c>
       <c r="T36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U36">
         <v>6</v>
@@ -3963,15 +4100,18 @@
         <v>22.49</v>
       </c>
       <c r="W36" s="3">
+        <f>V36*U36</f>
         <v>134.94</v>
       </c>
       <c r="X36">
         <v>6.98</v>
       </c>
       <c r="Y36" s="3">
+        <f>W36*X36/100</f>
         <v>9.4188</v>
       </c>
       <c r="Z36" s="3">
+        <f>W36+Y36</f>
         <v>144.3588</v>
       </c>
     </row>
@@ -4053,6 +4193,7 @@
         <v>0.15</v>
       </c>
       <c r="Q37" s="3">
+        <f>P37*B37</f>
         <v>0.15</v>
       </c>
       <c r="R37">
@@ -4073,15 +4214,18 @@
         <v>0.15</v>
       </c>
       <c r="W37" s="3">
+        <f>V37*U37</f>
         <v>0.45</v>
       </c>
       <c r="X37">
         <v>10</v>
       </c>
       <c r="Y37" s="3">
+        <f>W37*X37/100</f>
         <v>0.045</v>
       </c>
       <c r="Z37" s="3">
+        <f>W37+Y37</f>
         <v>0.495</v>
       </c>
     </row>
@@ -4159,6 +4303,7 @@
         <v>0.43</v>
       </c>
       <c r="Q38" s="3">
+        <f>P38*B38</f>
         <v>1.72</v>
       </c>
       <c r="R38">
@@ -4170,7 +4315,7 @@
         </is>
       </c>
       <c r="T38">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U38">
         <v>12</v>
@@ -4179,15 +4324,18 @@
         <v>0.302</v>
       </c>
       <c r="W38" s="3">
+        <f>V38*U38</f>
         <v>3.624</v>
       </c>
       <c r="X38">
         <v>7.91</v>
       </c>
       <c r="Y38" s="3">
+        <f>W38*X38/100</f>
         <v>0.2867</v>
       </c>
       <c r="Z38" s="3">
+        <f>W38+Y38</f>
         <v>3.9107</v>
       </c>
     </row>
@@ -4269,6 +4417,7 @@
         <v>0.11</v>
       </c>
       <c r="Q39" s="3">
+        <f>P39*B39</f>
         <v>0.66</v>
       </c>
       <c r="R39">
@@ -4280,7 +4429,7 @@
         </is>
       </c>
       <c r="T39">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="U39">
         <v>18</v>
@@ -4289,15 +4438,18 @@
         <v>0.102</v>
       </c>
       <c r="W39" s="3">
+        <f>V39*U39</f>
         <v>1.836</v>
       </c>
       <c r="X39">
         <v>0</v>
       </c>
       <c r="Y39" s="3">
+        <f>W39*X39/100</f>
         <v>0</v>
       </c>
       <c r="Z39" s="3">
+        <f>W39+Y39</f>
         <v>1.836</v>
       </c>
     </row>
@@ -4379,6 +4531,7 @@
         <v>0.23</v>
       </c>
       <c r="Q40" s="3">
+        <f>P40*B40</f>
         <v>3.22</v>
       </c>
       <c r="R40">
@@ -4390,7 +4543,7 @@
         </is>
       </c>
       <c r="T40">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="U40">
         <v>42</v>
@@ -4399,15 +4552,18 @@
         <v>0.096</v>
       </c>
       <c r="W40" s="3">
+        <f>V40*U40</f>
         <v>4.032</v>
       </c>
       <c r="X40">
         <v>7.83</v>
       </c>
       <c r="Y40" s="3">
+        <f>W40*X40/100</f>
         <v>0.3157</v>
       </c>
       <c r="Z40" s="3">
+        <f>W40+Y40</f>
         <v>4.3477</v>
       </c>
     </row>
@@ -4481,6 +4637,7 @@
         <v>0.19</v>
       </c>
       <c r="Q41" s="3">
+        <f>P41*B41</f>
         <v>0.57</v>
       </c>
       <c r="R41">
@@ -4492,7 +4649,7 @@
         </is>
       </c>
       <c r="T41">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U41">
         <v>10</v>
@@ -4501,15 +4658,18 @@
         <v>0.163</v>
       </c>
       <c r="W41" s="3">
+        <f>V41*U41</f>
         <v>1.63</v>
       </c>
       <c r="X41">
         <v>0</v>
       </c>
       <c r="Y41" s="3">
+        <f>W41*X41/100</f>
         <v>0</v>
       </c>
       <c r="Z41" s="3">
+        <f>W41+Y41</f>
         <v>1.63</v>
       </c>
     </row>
@@ -4591,6 +4751,7 @@
         <v>0.1</v>
       </c>
       <c r="Q42" s="3">
+        <f>P42*B42</f>
         <v>0.1</v>
       </c>
       <c r="R42">
@@ -4611,15 +4772,18 @@
         <v>0.016</v>
       </c>
       <c r="W42" s="3">
+        <f>V42*U42</f>
         <v>0.16</v>
       </c>
       <c r="X42">
         <v>0</v>
       </c>
       <c r="Y42" s="3">
+        <f>W42*X42/100</f>
         <v>0</v>
       </c>
       <c r="Z42" s="3">
+        <f>W42+Y42</f>
         <v>0.16</v>
       </c>
     </row>
@@ -4701,6 +4865,7 @@
         <v>0.28</v>
       </c>
       <c r="Q43" s="3">
+        <f>P43*B43</f>
         <v>0.28</v>
       </c>
       <c r="R43">
@@ -4721,15 +4886,18 @@
         <v>0.28</v>
       </c>
       <c r="W43" s="3">
+        <f>V43*U43</f>
         <v>0.84</v>
       </c>
       <c r="X43">
         <v>0</v>
       </c>
       <c r="Y43" s="3">
+        <f>W43*X43/100</f>
         <v>0</v>
       </c>
       <c r="Z43" s="3">
+        <f>W43+Y43</f>
         <v>0.84</v>
       </c>
     </row>
@@ -4811,6 +4979,7 @@
         <v>0.16</v>
       </c>
       <c r="Q44" s="3">
+        <f>P44*B44</f>
         <v>0.16</v>
       </c>
       <c r="R44">
@@ -4831,15 +5000,18 @@
         <v>0.16</v>
       </c>
       <c r="W44" s="3">
+        <f>V44*U44</f>
         <v>0.48</v>
       </c>
       <c r="X44">
         <v>0</v>
       </c>
       <c r="Y44" s="3">
+        <f>W44*X44/100</f>
         <v>0</v>
       </c>
       <c r="Z44" s="3">
+        <f>W44+Y44</f>
         <v>0.48</v>
       </c>
     </row>
@@ -4917,6 +5089,7 @@
         <v>0.9</v>
       </c>
       <c r="Q45" s="3">
+        <f>P45*B45</f>
         <v>4.5</v>
       </c>
       <c r="R45">
@@ -4928,7 +5101,7 @@
         </is>
       </c>
       <c r="T45">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U45">
         <v>15</v>
@@ -4937,15 +5110,18 @@
         <v>0.643</v>
       </c>
       <c r="W45" s="3">
+        <f>V45*U45</f>
         <v>9.645</v>
       </c>
       <c r="X45">
         <v>8</v>
       </c>
       <c r="Y45" s="3">
+        <f>W45*X45/100</f>
         <v>0.7716</v>
       </c>
       <c r="Z45" s="3">
+        <f>W45+Y45</f>
         <v>10.4166</v>
       </c>
     </row>
@@ -5027,6 +5203,7 @@
         <v>0.1</v>
       </c>
       <c r="Q46" s="3">
+        <f>P46*B46</f>
         <v>0.1</v>
       </c>
       <c r="R46">
@@ -5047,15 +5224,18 @@
         <v>0.016</v>
       </c>
       <c r="W46" s="3">
+        <f>V46*U46</f>
         <v>0.16</v>
       </c>
       <c r="X46">
         <v>8</v>
       </c>
       <c r="Y46" s="3">
+        <f>W46*X46/100</f>
         <v>0.0128</v>
       </c>
       <c r="Z46" s="3">
+        <f>W46+Y46</f>
         <v>0.1728</v>
       </c>
     </row>
@@ -5133,6 +5313,7 @@
         <v>0.29</v>
       </c>
       <c r="Q47" s="3">
+        <f>P47*B47</f>
         <v>0.87</v>
       </c>
       <c r="R47">
@@ -5144,7 +5325,7 @@
         </is>
       </c>
       <c r="T47">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U47">
         <v>10</v>
@@ -5153,15 +5334,18 @@
         <v>0.195</v>
       </c>
       <c r="W47" s="3">
+        <f>V47*U47</f>
         <v>1.95</v>
       </c>
       <c r="X47">
         <v>7.93</v>
       </c>
       <c r="Y47" s="3">
+        <f>W47*X47/100</f>
         <v>0.1546</v>
       </c>
       <c r="Z47" s="3">
+        <f>W47+Y47</f>
         <v>2.1046</v>
       </c>
     </row>
@@ -5239,6 +5423,7 @@
         <v>1.71</v>
       </c>
       <c r="Q48" s="3">
+        <f>P48*B48</f>
         <v>1.71</v>
       </c>
       <c r="R48">
@@ -5259,15 +5444,18 @@
         <v>1.71</v>
       </c>
       <c r="W48" s="3">
+        <f>V48*U48</f>
         <v>5.13</v>
       </c>
       <c r="X48">
         <v>0</v>
       </c>
       <c r="Y48" s="3">
+        <f>W48*X48/100</f>
         <v>0</v>
       </c>
       <c r="Z48" s="3">
+        <f>W48+Y48</f>
         <v>5.13</v>
       </c>
     </row>
@@ -5345,6 +5533,7 @@
         <v>1.38</v>
       </c>
       <c r="Q49" s="3">
+        <f>P49*B49</f>
         <v>2.76</v>
       </c>
       <c r="R49">
@@ -5356,7 +5545,7 @@
         </is>
       </c>
       <c r="T49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U49">
         <v>6</v>
@@ -5365,15 +5554,18 @@
         <v>1.38</v>
       </c>
       <c r="W49" s="3">
+        <f>V49*U49</f>
         <v>8.28</v>
       </c>
       <c r="X49">
         <v>0</v>
       </c>
       <c r="Y49" s="3">
+        <f>W49*X49/100</f>
         <v>0</v>
       </c>
       <c r="Z49" s="3">
+        <f>W49+Y49</f>
         <v>8.28</v>
       </c>
     </row>
@@ -5455,6 +5647,7 @@
         <v>0.1</v>
       </c>
       <c r="Q50" s="3">
+        <f>P50*B50</f>
         <v>0.4</v>
       </c>
       <c r="R50">
@@ -5466,7 +5659,7 @@
         </is>
       </c>
       <c r="T50">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U50">
         <v>12</v>
@@ -5475,15 +5668,18 @@
         <v>0.012</v>
       </c>
       <c r="W50" s="3">
+        <f>V50*U50</f>
         <v>0.144</v>
       </c>
       <c r="X50">
         <v>0</v>
       </c>
       <c r="Y50" s="3">
+        <f>W50*X50/100</f>
         <v>0</v>
       </c>
       <c r="Z50" s="3">
+        <f>W50+Y50</f>
         <v>0.144</v>
       </c>
     </row>
@@ -5565,6 +5761,7 @@
         <v>0.39</v>
       </c>
       <c r="Q51" s="3">
+        <f>P51*B51</f>
         <v>0.78</v>
       </c>
       <c r="R51">
@@ -5576,7 +5773,7 @@
         </is>
       </c>
       <c r="T51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U51">
         <v>10</v>
@@ -5585,15 +5782,18 @@
         <v>0.17</v>
       </c>
       <c r="W51" s="3">
+        <f>V51*U51</f>
         <v>1.7</v>
       </c>
       <c r="X51">
         <v>7.95</v>
       </c>
       <c r="Y51" s="3">
+        <f>W51*X51/100</f>
         <v>0.1351</v>
       </c>
       <c r="Z51" s="3">
+        <f>W51+Y51</f>
         <v>1.8351</v>
       </c>
     </row>
@@ -5671,6 +5871,7 @@
         <v>0.16</v>
       </c>
       <c r="Q52" s="3">
+        <f>P52*B52</f>
         <v>0.16</v>
       </c>
       <c r="R52">
@@ -5691,15 +5892,18 @@
         <v>0.16</v>
       </c>
       <c r="W52" s="3">
+        <f>V52*U52</f>
         <v>0.48</v>
       </c>
       <c r="X52">
         <v>35</v>
       </c>
       <c r="Y52" s="3">
+        <f>W52*X52/100</f>
         <v>0.168</v>
       </c>
       <c r="Z52" s="3">
+        <f>W52+Y52</f>
         <v>0.648</v>
       </c>
     </row>
@@ -5777,6 +5981,7 @@
         <v>17.13</v>
       </c>
       <c r="Q53" s="3">
+        <f>P53*B53</f>
         <v>17.13</v>
       </c>
       <c r="R53">
@@ -5797,15 +6002,18 @@
         <v>17.13</v>
       </c>
       <c r="W53" s="3">
+        <f>V53*U53</f>
         <v>51.39</v>
       </c>
       <c r="X53">
         <v>0</v>
       </c>
       <c r="Y53" s="3">
+        <f>W53*X53/100</f>
         <v>0</v>
       </c>
       <c r="Z53" s="3">
+        <f>W53+Y53</f>
         <v>51.39</v>
       </c>
     </row>
@@ -5879,6 +6087,7 @@
         <v>2.99</v>
       </c>
       <c r="Q54" s="3">
+        <f>P54*B54</f>
         <v>2.99</v>
       </c>
       <c r="R54">
@@ -5899,15 +6108,18 @@
         <v>2.99</v>
       </c>
       <c r="W54" s="3">
+        <f>V54*U54</f>
         <v>8.97</v>
       </c>
       <c r="X54">
         <v>0</v>
       </c>
       <c r="Y54" s="3">
+        <f>W54*X54/100</f>
         <v>0</v>
       </c>
       <c r="Z54" s="3">
+        <f>W54+Y54</f>
         <v>8.97</v>
       </c>
     </row>
@@ -5989,6 +6201,7 @@
         <v>0.1</v>
       </c>
       <c r="Q55" s="3">
+        <f>P55*B55</f>
         <v>0.1</v>
       </c>
       <c r="R55">
@@ -6009,15 +6222,18 @@
         <v>0.017</v>
       </c>
       <c r="W55" s="3">
+        <f>V55*U55</f>
         <v>0.17</v>
       </c>
       <c r="X55">
         <v>30</v>
       </c>
       <c r="Y55" s="3">
+        <f>W55*X55/100</f>
         <v>0.051</v>
       </c>
       <c r="Z55" s="3">
+        <f>W55+Y55</f>
         <v>0.221</v>
       </c>
     </row>
@@ -6099,6 +6315,7 @@
         <v>0.23</v>
       </c>
       <c r="Q56" s="3">
+        <f>P56*B56</f>
         <v>0.69</v>
       </c>
       <c r="R56">
@@ -6110,7 +6327,7 @@
         </is>
       </c>
       <c r="T56">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U56">
         <v>10</v>
@@ -6119,15 +6336,18 @@
         <v>0.081</v>
       </c>
       <c r="W56" s="3">
+        <f>V56*U56</f>
         <v>0.81</v>
       </c>
       <c r="X56">
         <v>7.83</v>
       </c>
       <c r="Y56" s="3">
+        <f>W56*X56/100</f>
         <v>0.0634</v>
       </c>
       <c r="Z56" s="3">
+        <f>W56+Y56</f>
         <v>0.8734</v>
       </c>
     </row>
@@ -6205,6 +6425,7 @@
         <v>2.75</v>
       </c>
       <c r="Q57" s="3">
+        <f>P57*B57</f>
         <v>2.75</v>
       </c>
       <c r="R57">
@@ -6225,15 +6446,18 @@
         <v>2.75</v>
       </c>
       <c r="W57" s="3">
+        <f>V57*U57</f>
         <v>8.25</v>
       </c>
       <c r="X57">
         <v>0</v>
       </c>
       <c r="Y57" s="3">
+        <f>W57*X57/100</f>
         <v>0</v>
       </c>
       <c r="Z57" s="3">
+        <f>W57+Y57</f>
         <v>8.25</v>
       </c>
     </row>
@@ -6315,6 +6539,7 @@
         <v>0.1</v>
       </c>
       <c r="Q58" s="3">
+        <f>P58*B58</f>
         <v>0.1</v>
       </c>
       <c r="R58">
@@ -6335,15 +6560,18 @@
         <v>0.1</v>
       </c>
       <c r="W58" s="3">
+        <f>V58*U58</f>
         <v>0.3</v>
       </c>
       <c r="X58">
         <v>8</v>
       </c>
       <c r="Y58" s="3">
+        <f>W58*X58/100</f>
         <v>0.024</v>
       </c>
       <c r="Z58" s="3">
+        <f>W58+Y58</f>
         <v>0.324</v>
       </c>
     </row>
@@ -6425,6 +6653,7 @@
         <v>0.1</v>
       </c>
       <c r="Q59" s="3">
+        <f>P59*B59</f>
         <v>0.1</v>
       </c>
       <c r="R59">
@@ -6445,15 +6674,18 @@
         <v>0.021</v>
       </c>
       <c r="W59" s="3">
+        <f>V59*U59</f>
         <v>0.21</v>
       </c>
       <c r="X59">
         <v>8</v>
       </c>
       <c r="Y59" s="3">
+        <f>W59*X59/100</f>
         <v>0.0168</v>
       </c>
       <c r="Z59" s="3">
+        <f>W59+Y59</f>
         <v>0.2268</v>
       </c>
     </row>
@@ -6527,6 +6759,7 @@
         <v>5.75</v>
       </c>
       <c r="Q60" s="3">
+        <f>P60*B60</f>
         <v>11.5</v>
       </c>
       <c r="R60">
@@ -6538,7 +6771,7 @@
         </is>
       </c>
       <c r="T60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U60">
         <v>6</v>
@@ -6547,15 +6780,18 @@
         <v>5.75</v>
       </c>
       <c r="W60" s="3">
+        <f>V60*U60</f>
         <v>34.5</v>
       </c>
       <c r="X60">
         <v>8</v>
       </c>
       <c r="Y60" s="3">
+        <f>W60*X60/100</f>
         <v>2.76</v>
       </c>
       <c r="Z60" s="3">
+        <f>W60+Y60</f>
         <v>37.26</v>
       </c>
     </row>
@@ -6637,6 +6873,7 @@
         <v>0.1</v>
       </c>
       <c r="Q61" s="3">
+        <f>P61*B61</f>
         <v>0.1</v>
       </c>
       <c r="R61">
@@ -6657,15 +6894,18 @@
         <v>0.012</v>
       </c>
       <c r="W61" s="3">
+        <f>V61*U61</f>
         <v>0.12</v>
       </c>
       <c r="X61">
         <v>0</v>
       </c>
       <c r="Y61" s="3">
+        <f>W61*X61/100</f>
         <v>0</v>
       </c>
       <c r="Z61" s="3">
+        <f>W61+Y61</f>
         <v>0.12</v>
       </c>
     </row>
@@ -6739,6 +6979,7 @@
         <v>1.1</v>
       </c>
       <c r="Q62" s="3">
+        <f>P62*B62</f>
         <v>1.1</v>
       </c>
       <c r="R62">
@@ -6759,15 +7000,18 @@
         <v>1.1</v>
       </c>
       <c r="W62" s="3">
+        <f>V62*U62</f>
         <v>3.3</v>
       </c>
       <c r="X62">
         <v>8</v>
       </c>
       <c r="Y62" s="3">
+        <f>W62*X62/100</f>
         <v>0.264</v>
       </c>
       <c r="Z62" s="3">
+        <f>W62+Y62</f>
         <v>3.564</v>
       </c>
     </row>
@@ -6845,6 +7089,7 @@
         <v>2.44</v>
       </c>
       <c r="Q63" s="3">
+        <f>P63*B63</f>
         <v>2.44</v>
       </c>
       <c r="R63">
@@ -6865,15 +7110,18 @@
         <v>2.44</v>
       </c>
       <c r="W63" s="3">
+        <f>V63*U63</f>
         <v>7.32</v>
       </c>
       <c r="X63">
         <v>0</v>
       </c>
       <c r="Y63" s="3">
+        <f>W63*X63/100</f>
         <v>0</v>
       </c>
       <c r="Z63" s="3">
+        <f>W63+Y63</f>
         <v>7.32</v>
       </c>
     </row>
@@ -6955,6 +7203,7 @@
         <v>0.1</v>
       </c>
       <c r="Q64" s="3">
+        <f>P64*B64</f>
         <v>0.1</v>
       </c>
       <c r="R64">
@@ -6975,15 +7224,18 @@
         <v>0.016</v>
       </c>
       <c r="W64" s="3">
+        <f>V64*U64</f>
         <v>0.16</v>
       </c>
       <c r="X64">
         <v>0</v>
       </c>
       <c r="Y64" s="3">
+        <f>W64*X64/100</f>
         <v>0</v>
       </c>
       <c r="Z64" s="3">
+        <f>W64+Y64</f>
         <v>0.16</v>
       </c>
     </row>
@@ -7065,6 +7317,7 @@
         <v>0.1</v>
       </c>
       <c r="Q65" s="3">
+        <f>P65*B65</f>
         <v>0.1</v>
       </c>
       <c r="R65">
@@ -7085,15 +7338,18 @@
         <v>0.013</v>
       </c>
       <c r="W65" s="3">
+        <f>V65*U65</f>
         <v>0.13</v>
       </c>
       <c r="X65">
         <v>10</v>
       </c>
       <c r="Y65" s="3">
+        <f>W65*X65/100</f>
         <v>0.013</v>
       </c>
       <c r="Z65" s="3">
+        <f>W65+Y65</f>
         <v>0.143</v>
       </c>
     </row>
@@ -7175,6 +7431,7 @@
         <v>0.1</v>
       </c>
       <c r="Q66" s="3">
+        <f>P66*B66</f>
         <v>0.1</v>
       </c>
       <c r="R66">
@@ -7195,15 +7452,18 @@
         <v>0.023</v>
       </c>
       <c r="W66" s="3">
+        <f>V66*U66</f>
         <v>0.23</v>
       </c>
       <c r="X66">
         <v>8</v>
       </c>
       <c r="Y66" s="3">
+        <f>W66*X66/100</f>
         <v>0.0184</v>
       </c>
       <c r="Z66" s="3">
+        <f>W66+Y66</f>
         <v>0.2484</v>
       </c>
     </row>
@@ -7285,6 +7545,7 @@
         <v>0.1</v>
       </c>
       <c r="Q67" s="3">
+        <f>P67*B67</f>
         <v>0.1</v>
       </c>
       <c r="R67">
@@ -7305,15 +7566,18 @@
         <v>0.009</v>
       </c>
       <c r="W67" s="3">
+        <f>V67*U67</f>
         <v>0.09</v>
       </c>
       <c r="X67">
         <v>8</v>
       </c>
       <c r="Y67" s="3">
+        <f>W67*X67/100</f>
         <v>0.0072</v>
       </c>
       <c r="Z67" s="3">
+        <f>W67+Y67</f>
         <v>0.0972</v>
       </c>
     </row>
@@ -7391,6 +7655,7 @@
         <v>0.79</v>
       </c>
       <c r="Q68" s="3">
+        <f>P68*B68</f>
         <v>0.79</v>
       </c>
       <c r="R68">
@@ -7411,15 +7676,18 @@
         <v>0.79</v>
       </c>
       <c r="W68" s="3">
+        <f>V68*U68</f>
         <v>2.37</v>
       </c>
       <c r="X68">
         <v>0</v>
       </c>
       <c r="Y68" s="3">
+        <f>W68*X68/100</f>
         <v>0</v>
       </c>
       <c r="Z68" s="3">
+        <f>W68+Y68</f>
         <v>2.37</v>
       </c>
     </row>
@@ -7497,6 +7765,7 @@
         <v>6.99</v>
       </c>
       <c r="Q69" s="3">
+        <f>P69*B69</f>
         <v>6.99</v>
       </c>
       <c r="R69">
@@ -7517,15 +7786,18 @@
         <v>6.99</v>
       </c>
       <c r="W69" s="3">
+        <f>V69*U69</f>
         <v>20.97</v>
       </c>
       <c r="X69">
         <v>0</v>
       </c>
       <c r="Y69" s="3">
+        <f>W69*X69/100</f>
         <v>0</v>
       </c>
       <c r="Z69" s="3">
+        <f>W69+Y69</f>
         <v>20.97</v>
       </c>
     </row>
@@ -7607,6 +7879,7 @@
         <v>0.1</v>
       </c>
       <c r="Q70" s="3">
+        <f>P70*B70</f>
         <v>0.2</v>
       </c>
       <c r="R70">
@@ -7618,7 +7891,7 @@
         </is>
       </c>
       <c r="T70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U70">
         <v>10</v>
@@ -7627,15 +7900,18 @@
         <v>0.012</v>
       </c>
       <c r="W70" s="3">
+        <f>V70*U70</f>
         <v>0.12</v>
       </c>
       <c r="X70">
         <v>0</v>
       </c>
       <c r="Y70" s="3">
+        <f>W70*X70/100</f>
         <v>0</v>
       </c>
       <c r="Z70" s="3">
+        <f>W70+Y70</f>
         <v>0.12</v>
       </c>
     </row>
@@ -7713,6 +7989,7 @@
         <v>0.16</v>
       </c>
       <c r="Q71" s="3">
+        <f>P71*B71</f>
         <v>0.16</v>
       </c>
       <c r="R71">
@@ -7733,15 +8010,18 @@
         <v>0.16</v>
       </c>
       <c r="W71" s="3">
+        <f>V71*U71</f>
         <v>0.48</v>
       </c>
       <c r="X71">
         <v>35</v>
       </c>
       <c r="Y71" s="3">
+        <f>W71*X71/100</f>
         <v>0.168</v>
       </c>
       <c r="Z71" s="3">
+        <f>W71+Y71</f>
         <v>0.648</v>
       </c>
     </row>
@@ -7823,6 +8103,7 @@
         <v>0.1</v>
       </c>
       <c r="Q72" s="3">
+        <f>P72*B72</f>
         <v>0.1</v>
       </c>
       <c r="R72">
@@ -7843,15 +8124,18 @@
         <v>0.011</v>
       </c>
       <c r="W72" s="3">
+        <f>V72*U72</f>
         <v>0.11</v>
       </c>
       <c r="X72">
         <v>0</v>
       </c>
       <c r="Y72" s="3">
+        <f>W72*X72/100</f>
         <v>0</v>
       </c>
       <c r="Z72" s="3">
+        <f>W72+Y72</f>
         <v>0.11</v>
       </c>
     </row>
@@ -7929,6 +8213,7 @@
         <v>0.22</v>
       </c>
       <c r="Q73" s="3">
+        <f>P73*B73</f>
         <v>2.64</v>
       </c>
       <c r="R73">
@@ -7940,7 +8225,7 @@
         </is>
       </c>
       <c r="T73">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="U73">
         <v>36</v>
@@ -7949,15 +8234,18 @@
         <v>0.131</v>
       </c>
       <c r="W73" s="3">
+        <f>V73*U73</f>
         <v>4.716</v>
       </c>
       <c r="X73">
         <v>0</v>
       </c>
       <c r="Y73" s="3">
+        <f>W73*X73/100</f>
         <v>0</v>
       </c>
       <c r="Z73" s="3">
+        <f>W73+Y73</f>
         <v>4.716</v>
       </c>
     </row>
@@ -8039,6 +8327,7 @@
         <v>0.28</v>
       </c>
       <c r="Q74" s="3">
+        <f>P74*B74</f>
         <v>0.28</v>
       </c>
       <c r="R74">
@@ -8059,15 +8348,18 @@
         <v>0.28</v>
       </c>
       <c r="W74" s="3">
+        <f>V74*U74</f>
         <v>0.84</v>
       </c>
       <c r="X74">
         <v>0</v>
       </c>
       <c r="Y74" s="3">
+        <f>W74*X74/100</f>
         <v>0</v>
       </c>
       <c r="Z74" s="3">
+        <f>W74+Y74</f>
         <v>0.84</v>
       </c>
     </row>
@@ -8149,6 +8441,7 @@
         <v>0.28</v>
       </c>
       <c r="Q75" s="3">
+        <f>P75*B75</f>
         <v>0.28</v>
       </c>
       <c r="R75">
@@ -8169,15 +8462,18 @@
         <v>0.28</v>
       </c>
       <c r="W75" s="3">
+        <f>V75*U75</f>
         <v>0.84</v>
       </c>
       <c r="X75">
         <v>0</v>
       </c>
       <c r="Y75" s="3">
+        <f>W75*X75/100</f>
         <v>0</v>
       </c>
       <c r="Z75" s="3">
+        <f>W75+Y75</f>
         <v>0.84</v>
       </c>
     </row>
@@ -8255,6 +8551,7 @@
         <v>0.36</v>
       </c>
       <c r="Q76" s="3">
+        <f>P76*B76</f>
         <v>2.52</v>
       </c>
       <c r="R76">
@@ -8266,7 +8563,7 @@
         </is>
       </c>
       <c r="T76">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="U76">
         <v>21</v>
@@ -8275,15 +8572,18 @@
         <v>0.246</v>
       </c>
       <c r="W76" s="3">
+        <f>V76*U76</f>
         <v>5.166</v>
       </c>
       <c r="X76">
         <v>0</v>
       </c>
       <c r="Y76" s="3">
+        <f>W76*X76/100</f>
         <v>0</v>
       </c>
       <c r="Z76" s="3">
+        <f>W76+Y76</f>
         <v>5.166</v>
       </c>
     </row>
@@ -8365,6 +8665,7 @@
         <v>0.12</v>
       </c>
       <c r="Q77" s="3">
+        <f>P77*B77</f>
         <v>0.12</v>
       </c>
       <c r="R77">
@@ -8385,15 +8686,18 @@
         <v>0.12</v>
       </c>
       <c r="W77" s="3">
+        <f>V77*U77</f>
         <v>0.36</v>
       </c>
       <c r="X77">
         <v>8.33</v>
       </c>
       <c r="Y77" s="3">
+        <f>W77*X77/100</f>
         <v>0.03</v>
       </c>
       <c r="Z77" s="3">
+        <f>W77+Y77</f>
         <v>0.39</v>
       </c>
     </row>
@@ -8471,6 +8775,7 @@
         <v>0.5</v>
       </c>
       <c r="Q78" s="3">
+        <f>P78*B78</f>
         <v>0.5</v>
       </c>
       <c r="R78">
@@ -8491,15 +8796,18 @@
         <v>0.5</v>
       </c>
       <c r="W78" s="3">
+        <f>V78*U78</f>
         <v>1.5</v>
       </c>
       <c r="X78">
         <v>30</v>
       </c>
       <c r="Y78" s="3">
+        <f>W78*X78/100</f>
         <v>0.45</v>
       </c>
       <c r="Z78" s="3">
+        <f>W78+Y78</f>
         <v>1.95</v>
       </c>
     </row>
@@ -8577,6 +8885,7 @@
         <v>0.63</v>
       </c>
       <c r="Q79" s="3">
+        <f>P79*B79</f>
         <v>1.26</v>
       </c>
       <c r="R79">
@@ -8588,7 +8897,7 @@
         </is>
       </c>
       <c r="T79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U79">
         <v>6</v>
@@ -8597,15 +8906,18 @@
         <v>0.63</v>
       </c>
       <c r="W79" s="3">
+        <f>V79*U79</f>
         <v>3.78</v>
       </c>
       <c r="X79">
         <v>0</v>
       </c>
       <c r="Y79" s="3">
+        <f>W79*X79/100</f>
         <v>0</v>
       </c>
       <c r="Z79" s="3">
+        <f>W79+Y79</f>
         <v>3.78</v>
       </c>
     </row>
@@ -8687,6 +8999,7 @@
         <v>0.1</v>
       </c>
       <c r="Q80" s="3">
+        <f>P80*B80</f>
         <v>0.3</v>
       </c>
       <c r="R80">
@@ -8698,7 +9011,7 @@
         </is>
       </c>
       <c r="T80">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U80">
         <v>10</v>
@@ -8707,15 +9020,18 @@
         <v>0.029</v>
       </c>
       <c r="W80" s="3">
+        <f>V80*U80</f>
         <v>0.29</v>
       </c>
       <c r="X80">
         <v>0</v>
       </c>
       <c r="Y80" s="3">
+        <f>W80*X80/100</f>
         <v>0</v>
       </c>
       <c r="Z80" s="3">
+        <f>W80+Y80</f>
         <v>0.29</v>
       </c>
     </row>
@@ -8797,6 +9113,7 @@
         <v>0.1</v>
       </c>
       <c r="Q81" s="3">
+        <f>P81*B81</f>
         <v>0.1</v>
       </c>
       <c r="R81">
@@ -8817,15 +9134,18 @@
         <v>0.012</v>
       </c>
       <c r="W81" s="3">
+        <f>V81*U81</f>
         <v>0.12</v>
       </c>
       <c r="X81">
         <v>0</v>
       </c>
       <c r="Y81" s="3">
+        <f>W81*X81/100</f>
         <v>0</v>
       </c>
       <c r="Z81" s="3">
+        <f>W81+Y81</f>
         <v>0.12</v>
       </c>
     </row>
@@ -8899,6 +9219,7 @@
         <v>0.84</v>
       </c>
       <c r="Q82" s="3">
+        <f>P82*B82</f>
         <v>1.68</v>
       </c>
       <c r="R82">
@@ -8910,7 +9231,7 @@
         </is>
       </c>
       <c r="T82">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U82">
         <v>6</v>
@@ -8919,15 +9240,18 @@
         <v>0.84</v>
       </c>
       <c r="W82" s="3">
+        <f>V82*U82</f>
         <v>5.04</v>
       </c>
       <c r="X82">
         <v>7.98</v>
       </c>
       <c r="Y82" s="3">
+        <f>W82*X82/100</f>
         <v>0.4022</v>
       </c>
       <c r="Z82" s="3">
+        <f>W82+Y82</f>
         <v>5.4422</v>
       </c>
     </row>
@@ -9009,6 +9333,7 @@
         <v>0.1</v>
       </c>
       <c r="Q83" s="3">
+        <f>P83*B83</f>
         <v>0.1</v>
       </c>
       <c r="R83">
@@ -9029,15 +9354,18 @@
         <v>0.016</v>
       </c>
       <c r="W83" s="3">
+        <f>V83*U83</f>
         <v>0.16</v>
       </c>
       <c r="X83">
         <v>0</v>
       </c>
       <c r="Y83" s="3">
+        <f>W83*X83/100</f>
         <v>0</v>
       </c>
       <c r="Z83" s="3">
+        <f>W83+Y83</f>
         <v>0.16</v>
       </c>
     </row>
@@ -9119,6 +9447,7 @@
         <v>0.19</v>
       </c>
       <c r="Q84" s="3">
+        <f>P84*B84</f>
         <v>0.19</v>
       </c>
       <c r="R84">
@@ -9139,15 +9468,18 @@
         <v>0.19</v>
       </c>
       <c r="W84" s="3">
+        <f>V84*U84</f>
         <v>0.57</v>
       </c>
       <c r="X84">
         <v>0</v>
       </c>
       <c r="Y84" s="3">
+        <f>W84*X84/100</f>
         <v>0</v>
       </c>
       <c r="Z84" s="3">
+        <f>W84+Y84</f>
         <v>0.57</v>
       </c>
     </row>
@@ -9221,6 +9553,7 @@
         <v>0.36</v>
       </c>
       <c r="Q85" s="3">
+        <f>P85*B85</f>
         <v>0.72</v>
       </c>
       <c r="R85">
@@ -9232,7 +9565,7 @@
         </is>
       </c>
       <c r="T85">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U85">
         <v>6</v>
@@ -9241,15 +9574,18 @@
         <v>0.36</v>
       </c>
       <c r="W85" s="3">
+        <f>V85*U85</f>
         <v>2.16</v>
       </c>
       <c r="X85">
         <v>8.06</v>
       </c>
       <c r="Y85" s="3">
+        <f>W85*X85/100</f>
         <v>0.1741</v>
       </c>
       <c r="Z85" s="3">
+        <f>W85+Y85</f>
         <v>2.3341</v>
       </c>
     </row>
@@ -9331,6 +9667,7 @@
         <v>0.29</v>
       </c>
       <c r="Q86" s="3">
+        <f>P86*B86</f>
         <v>0.29</v>
       </c>
       <c r="R86">
@@ -9351,15 +9688,18 @@
         <v>0.29</v>
       </c>
       <c r="W86" s="3">
+        <f>V86*U86</f>
         <v>0.87</v>
       </c>
       <c r="X86">
         <v>0</v>
       </c>
       <c r="Y86" s="3">
+        <f>W86*X86/100</f>
         <v>0</v>
       </c>
       <c r="Z86" s="3">
+        <f>W86+Y86</f>
         <v>0.87</v>
       </c>
     </row>
@@ -9441,6 +9781,7 @@
         <v>0.24</v>
       </c>
       <c r="Q87" s="3">
+        <f>P87*B87</f>
         <v>0.48</v>
       </c>
       <c r="R87">
@@ -9452,7 +9793,7 @@
         </is>
       </c>
       <c r="T87">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U87">
         <v>10</v>
@@ -9461,15 +9802,18 @@
         <v>0.06</v>
       </c>
       <c r="W87" s="3">
+        <f>V87*U87</f>
         <v>0.6</v>
       </c>
       <c r="X87">
         <v>0</v>
       </c>
       <c r="Y87" s="3">
+        <f>W87*X87/100</f>
         <v>0</v>
       </c>
       <c r="Z87" s="3">
+        <f>W87+Y87</f>
         <v>0.6</v>
       </c>
     </row>
@@ -9551,6 +9895,7 @@
         <v>0.16</v>
       </c>
       <c r="Q88" s="3">
+        <f>P88*B88</f>
         <v>0.16</v>
       </c>
       <c r="R88">
@@ -9571,15 +9916,18 @@
         <v>0.16</v>
       </c>
       <c r="W88" s="3">
+        <f>V88*U88</f>
         <v>0.48</v>
       </c>
       <c r="X88">
         <v>0</v>
       </c>
       <c r="Y88" s="3">
+        <f>W88*X88/100</f>
         <v>0</v>
       </c>
       <c r="Z88" s="3">
+        <f>W88+Y88</f>
         <v>0.48</v>
       </c>
     </row>
@@ -9661,6 +10009,7 @@
         <v>0.11</v>
       </c>
       <c r="Q89" s="3">
+        <f>P89*B89</f>
         <v>0.11</v>
       </c>
       <c r="R89">
@@ -9681,15 +10030,18 @@
         <v>0.11</v>
       </c>
       <c r="W89" s="3">
+        <f>V89*U89</f>
         <v>0.33</v>
       </c>
       <c r="X89">
         <v>0</v>
       </c>
       <c r="Y89" s="3">
+        <f>W89*X89/100</f>
         <v>0</v>
       </c>
       <c r="Z89" s="3">
+        <f>W89+Y89</f>
         <v>0.33</v>
       </c>
     </row>
@@ -9721,13 +10073,16 @@
       <c r="U90"/>
       <c r="V90"/>
       <c r="W90" s="4">
+        <f>SUM(W2:W89)</f>
         <v>886.825</v>
       </c>
       <c r="X90"/>
       <c r="Y90" s="4">
+        <f>SUM(Y2:Y89)</f>
         <v>57.8504</v>
       </c>
       <c r="Z90" s="4">
+        <f>SUM(Z2:Z89)</f>
         <v>944.6754</v>
       </c>
     </row>

</xml_diff>